<commit_message>
data: hourly update 2026-06-27 21:03Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-06-27.xlsx
+++ b/data/output/workbook/2026-06-27.xlsx
@@ -954,7 +954,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-27 15:33</t>
+          <t>2026-06-27 17:03</t>
         </is>
       </c>
     </row>
@@ -8240,37 +8240,37 @@
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Phoenix Mercury @ Toronto Tempo</t>
+          <t>Cincinnati Reds @ Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 179.5</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.6043749999999999</v>
+        <v>0.6714396396396396</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-153</v>
+        <v>-204</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>108</v>
+        <v>-122</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -8294,7 +8294,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 60.4% (fair -153). Your call.</t>
+          <t>Model 67.1% (fair -204). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -8311,7 +8311,7 @@
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Pittsburgh Pirates</t>
+          <t>Washington Nationals @ Baltimore Orioles</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
@@ -8321,22 +8321,22 @@
       </c>
       <c r="D8" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.6685819819819819</v>
+        <v>0.5857560975609757</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-202</v>
+        <v>-141</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>-122</v>
+        <v>105</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -8360,7 +8360,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 66.9% (fair -202). Your call.</t>
+          <t>Model 58.6% (fair -141). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -8392,17 +8392,17 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Over 165.5</t>
+          <t>Over 166.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.6033500000000001</v>
+        <v>0.5774509803921568</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-152</v>
+        <v>-137</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -8426,7 +8426,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 60.3% (fair -152). Your call.</t>
+          <t>Model 57.7% (fair -137). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -8443,12 +8443,12 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Washington Nationals @ Baltimore Orioles</t>
+          <t>Houston Astros @ Detroit Tigers</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
@@ -8458,17 +8458,17 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Over 9.5</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5857560975609757</v>
+        <v>0.5746</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-141</v>
+        <v>-135</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -8492,7 +8492,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 58.6% (fair -141). Your call.</t>
+          <t>Model 57.5% (fair -135). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -8504,37 +8504,37 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Pittsburgh Pirates</t>
+          <t>Kansas City Royals @ Chicago White Sox</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Over 9</t>
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.559656862745098</v>
+        <v>0.5866682926829269</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-127</v>
+        <v>-142</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>104</v>
+        <v>-105</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -8558,7 +8558,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 56.0% (fair -127). Your call.</t>
+          <t>Model 58.7% (fair -142). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -8570,37 +8570,37 @@
     <row r="12">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>Kansas City Royals @ Chicago White Sox</t>
+          <t>Cincinnati Reds @ Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="D12" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
-          <t>Over 9</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.5817512195121951</v>
+        <v>0.5560194174757281</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-139</v>
+        <v>-125</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>-105</v>
+        <v>106</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -8624,7 +8624,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 58.2% (fair -139). Your call.</t>
+          <t>Model 55.6% (fair -125). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -8651,19 +8651,19 @@
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Golden State Valkyries</t>
+          <t>Golden State Valkyries +1.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.578321568627451</v>
+        <v>0.5795450980392156</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-137</v>
+        <v>-138</v>
       </c>
       <c r="H13" s="15" t="n">
         <v>-104</v>
@@ -8690,7 +8690,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 57.8% (fair -137). Your call.</t>
+          <t>Model 58.0% (fair -138). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -8717,19 +8717,19 @@
       </c>
       <c r="D14" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Golden State Valkyries +1.5</t>
+          <t>Golden State Valkyries</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.576435294117647</v>
+        <v>0.578321568627451</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-136</v>
+        <v>-137</v>
       </c>
       <c r="H14" s="15" t="n">
         <v>-104</v>
@@ -8756,7 +8756,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 57.6% (fair -136). Your call.</t>
+          <t>Model 57.8% (fair -137). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -8773,7 +8773,7 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks @ Tampa Bay Rays</t>
+          <t>Seattle Mariners @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
@@ -8783,22 +8783,22 @@
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.5958069767441861</v>
+        <v>0.54375</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-147</v>
+        <v>-119</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>-115</v>
+        <v>108</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -8822,7 +8822,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 59.6% (fair -147). Your call.</t>
+          <t>Model 54.4% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -8839,32 +8839,32 @@
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>Las Vegas Aces @ Chicago Sky</t>
+          <t>Arizona Diamondbacks @ Tampa Bay Rays</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Chicago Sky +7.5</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.5767615384615384</v>
+        <v>0.5958069767441861</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-136</v>
+        <v>-147</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>-108</v>
+        <v>-115</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -8888,7 +8888,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -136). Your call.</t>
+          <t>Model 59.6% (fair -147). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -8905,12 +8905,12 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Washington Nationals @ Baltimore Orioles</t>
+          <t>Las Vegas Aces @ Chicago Sky</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -8920,17 +8920,17 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Baltimore Orioles -1.5</t>
+          <t>Chicago Sky +7.5</t>
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.5273809523809523</v>
+        <v>0.5767615384615384</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-112</v>
+        <v>-136</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>110</v>
+        <v>-108</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -8954,7 +8954,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 52.7% (fair -112). Your call.</t>
+          <t>Model 57.7% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -8981,22 +8981,22 @@
       </c>
       <c r="D18" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Baltimore Orioles -1.5</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.6854057034220533</v>
+        <v>0.5273809523809523</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-218</v>
+        <v>-112</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>-163</v>
+        <v>110</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -9020,7 +9020,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 68.5% (fair -218). Your call.</t>
+          <t>Model 52.7% (fair -112). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -9037,32 +9037,32 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Las Vegas Aces @ Chicago Sky</t>
+          <t>Washington Nationals @ Baltimore Orioles</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 178.5</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.55275</v>
+        <v>0.6854057034220533</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-124</v>
+        <v>-218</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>100</v>
+        <v>-163</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -9086,7 +9086,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 55.3% (fair -124). Your call.</t>
+          <t>Model 68.5% (fair -218). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -9103,12 +9103,12 @@
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>New York Liberty @ Golden State Valkyries</t>
+          <t>Las Vegas Aces @ Chicago Sky</t>
         </is>
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
@@ -9118,17 +9118,17 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Over 163.5</t>
+          <t>Over 178.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.5769238095238095</v>
+        <v>0.55275</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>-136</v>
+        <v>-124</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>-110</v>
+        <v>100</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -9152,7 +9152,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -136). Your call.</t>
+          <t>Model 55.3% (fair -124). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -9188,13 +9188,13 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.5621853658536585</v>
+        <v>0.55175</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>-128</v>
+        <v>-123</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>-105</v>
+        <v>100</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -9218,7 +9218,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 56.2% (fair -128). Your call.</t>
+          <t>Model 55.2% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -9235,32 +9235,32 @@
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>Seattle Mariners @ Cleveland Guardians</t>
+          <t>New York Liberty @ Golden State Valkyries</t>
         </is>
       </c>
       <c r="C22" s="20" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D22" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Over 163.5</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.54865</v>
+        <v>0.5769238095238095</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-122</v>
+        <v>-136</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -9284,7 +9284,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 54.9% (fair -122). Your call.</t>
+          <t>Model 57.7% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -9320,10 +9320,10 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.5612634146341464</v>
+        <v>0.5636707317073171</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>-128</v>
+        <v>-129</v>
       </c>
       <c r="H23" s="15" t="n">
         <v>-105</v>
@@ -9350,7 +9350,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 56.1% (fair -128). Your call.</t>
+          <t>Model 56.4% (fair -129). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -9386,7 +9386,7 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5517098039215687</v>
+        <v>0.5510470588235293</v>
       </c>
       <c r="G24" s="14" t="n">
         <v>-123</v>
@@ -9416,7 +9416,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 55.2% (fair -123). Your call.</t>
+          <t>Model 55.1% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -9560,37 +9560,37 @@
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>Seattle Mariners @ Cleveland Guardians</t>
+          <t>New York Yankees @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>23:20</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Under 9</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.6186806722689074</v>
+        <v>0.5172596153846154</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>-162</v>
+        <v>-107</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>-138</v>
+        <v>108</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -9614,7 +9614,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 61.9% (fair -162). Your call.</t>
+          <t>Model 51.7% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -9631,32 +9631,32 @@
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>Atlanta Braves @ San Francisco Giants</t>
+          <t>Colorado Rockies @ Minnesota Twins</t>
         </is>
       </c>
       <c r="C28" s="20" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>San Francisco Giants +1.5</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.6019565217391304</v>
+        <v>0.53585</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-151</v>
+        <v>-115</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>-130</v>
+        <v>100</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -9680,7 +9680,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 60.2% (fair -151). Your call.</t>
+          <t>Model 53.6% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -9692,17 +9692,17 @@
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>Kansas City Royals @ Chicago White Sox</t>
+          <t>Chicago Cubs @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
@@ -9712,17 +9712,17 @@
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.5935991189427313</v>
+        <v>0.6324196721311476</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-146</v>
+        <v>-172</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>-127</v>
+        <v>-144</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -9746,7 +9746,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 59.4% (fair -146). Your call.</t>
+          <t>Model 63.2% (fair -172). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -9923,10 +9923,10 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4448878923766816</v>
+        <v>0.4398206278026906</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="H5" s="15" t="n">
         <v>123</v>
@@ -9953,7 +9953,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 44.5% (fair +125). Your call.</t>
+          <t>Model 44.0% (fair +127). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -9989,10 +9989,10 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5551074889867842</v>
+        <v>0.560198678414097</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-125</v>
+        <v>-127</v>
       </c>
       <c r="H6" s="15" t="n">
         <v>-127</v>
@@ -10019,7 +10019,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 55.5% (fair -125). Your call.</t>
+          <t>Model 56.0% (fair -127). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -10055,10 +10055,10 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5043</v>
+        <v>0.5093</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-102</v>
+        <v>-104</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>125</v>
@@ -10085,7 +10085,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 50.4% (fair -102). Your call.</t>
+          <t>Model 50.9% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -10121,10 +10121,10 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4957</v>
+        <v>0.4907</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H8" s="15" t="n">
         <v>100</v>
@@ -10151,7 +10151,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 49.6% (fair +102). Your call.</t>
+          <t>Model 49.1% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -10187,10 +10187,10 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.3795769230769231</v>
+        <v>0.3830384615384615</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="H9" s="15" t="n">
         <v>160</v>
@@ -10217,7 +10217,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 38.0% (fair +163). Your call.</t>
+          <t>Model 38.3% (fair +161). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -10253,10 +10253,10 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.6204536121673004</v>
+        <v>0.6169828897338403</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-163</v>
+        <v>-161</v>
       </c>
       <c r="H10" s="15" t="n">
         <v>-163</v>
@@ -10283,7 +10283,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 62.0% (fair -163). Your call.</t>
+          <t>Model 61.7% (fair -161). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -10319,10 +10319,10 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.5328980392156862</v>
+        <v>0.5287686274509803</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-114</v>
+        <v>-112</v>
       </c>
       <c r="H11" s="15" t="n">
         <v>-104</v>
@@ -10349,7 +10349,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 53.3% (fair -114). Your call.</t>
+          <t>Model 52.9% (fair -112). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -10385,10 +10385,10 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.4671078431372549</v>
+        <v>0.4712254901960785</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H12" s="15" t="n">
         <v>104</v>
@@ -10415,7 +10415,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 46.7% (fair +114). Your call.</t>
+          <t>Model 47.1% (fair +112). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -10451,10 +10451,10 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5877</v>
+        <v>0.5897</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-143</v>
+        <v>-144</v>
       </c>
       <c r="H13" s="15" t="n">
         <v>117</v>
@@ -10481,7 +10481,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 58.8% (fair -143). Your call.</t>
+          <t>Model 59.0% (fair -144). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -10517,10 +10517,10 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4123</v>
+        <v>0.4103</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H14" s="15" t="n">
         <v>111</v>
@@ -10547,7 +10547,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 41.2% (fair +143). Your call.</t>
+          <t>Model 41.0% (fair +144). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -10583,10 +10583,10 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.2686</v>
+        <v>0.2759</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>272</v>
+        <v>262</v>
       </c>
       <c r="H15" s="15" t="n">
         <v>172</v>
@@ -10613,7 +10613,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 26.9% (fair +272). Your call.</t>
+          <t>Model 27.6% (fair +262). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -10649,10 +10649,10 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.7314000000000001</v>
+        <v>0.7241</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-272</v>
+        <v>-262</v>
       </c>
       <c r="H16" s="15" t="n">
         <v>156</v>
@@ -10679,7 +10679,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 73.1% (fair -272). Your call.</t>
+          <t>Model 72.4% (fair -262). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -11051,7 +11051,7 @@
         <v>-139</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>170</v>
+        <v>126</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -11111,13 +11111,13 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.44035</v>
+        <v>0.4439882352941176</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>100</v>
+        <v>-104</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -11141,7 +11141,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 44.0% (fair +127). Your call.</t>
+          <t>Model 44.4% (fair +125). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -11177,13 +11177,13 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.559656862745098</v>
+        <v>0.5560194174757281</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-127</v>
+        <v>-125</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -11207,7 +11207,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 56.0% (fair -127). Your call.</t>
+          <t>Model 55.6% (fair -125). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -11315,7 +11315,7 @@
         <v>189</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -11375,13 +11375,13 @@
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.4883870967741936</v>
+        <v>0.4857272727272727</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -11405,7 +11405,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 48.8% (fair +105). Your call.</t>
+          <t>Model 48.6% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -11441,13 +11441,13 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.5116363636363636</v>
+        <v>0.5142684684684684</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-105</v>
+        <v>-106</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>-120</v>
+        <v>-122</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -11471,7 +11471,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 51.2% (fair -105). Your call.</t>
+          <t>Model 51.4% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -11513,7 +11513,7 @@
         <v>217</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -11579,7 +11579,7 @@
         <v>-217</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="I30" s="13">
         <f>IF($H$30="","",IF($H$30&lt;0,-$H$30/(-$H$30+100),100/($H$30+100)))</f>
@@ -11711,7 +11711,7 @@
         <v>-240</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>-124</v>
+        <v>-129</v>
       </c>
       <c r="I32" s="13">
         <f>IF($H$32="","",IF($H$32&lt;0,-$H$32/(-$H$32+100),100/($H$32+100)))</f>
@@ -11777,7 +11777,7 @@
         <v>186</v>
       </c>
       <c r="H33" s="15" t="n">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="I33" s="13">
         <f>IF($H$33="","",IF($H$33&lt;0,-$H$33/(-$H$33+100),100/($H$33+100)))</f>
@@ -12107,7 +12107,7 @@
         <v>-115</v>
       </c>
       <c r="H38" s="15" t="n">
-        <v>-126</v>
+        <v>-130</v>
       </c>
       <c r="I38" s="13">
         <f>IF($H$38="","",IF($H$38&lt;0,-$H$38/(-$H$38+100),100/($H$38+100)))</f>
@@ -12299,10 +12299,10 @@
         </is>
       </c>
       <c r="F41" s="13" t="n">
-        <v>0.4975490196078431</v>
+        <v>0.5026</v>
       </c>
       <c r="G41" s="14" t="n">
-        <v>101</v>
+        <v>-101</v>
       </c>
       <c r="H41" s="15" t="n">
         <v>104</v>
@@ -12329,7 +12329,7 @@
       </c>
       <c r="N41" s="19" t="inlineStr">
         <is>
-          <t>Model 49.8% (fair +101). Your call.</t>
+          <t>Model 50.3% (fair -101). Your call.</t>
         </is>
       </c>
       <c r="O41" s="15" t="n"/>
@@ -12365,13 +12365,13 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.5024257425742574</v>
+        <v>0.4974</v>
       </c>
       <c r="G42" s="14" t="n">
-        <v>-101</v>
+        <v>101</v>
       </c>
       <c r="H42" s="15" t="n">
-        <v>-102</v>
+        <v>116</v>
       </c>
       <c r="I42" s="13">
         <f>IF($H$42="","",IF($H$42&lt;0,-$H$42/(-$H$42+100),100/($H$42+100)))</f>
@@ -12395,7 +12395,7 @@
       </c>
       <c r="N42" s="19" t="inlineStr">
         <is>
-          <t>Model 50.2% (fair -101). Your call.</t>
+          <t>Model 49.7% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O42" s="15" t="n"/>
@@ -12563,13 +12563,13 @@
         </is>
       </c>
       <c r="F45" s="13" t="n">
-        <v>0.4483251231527093</v>
+        <v>0.4489108910891089</v>
       </c>
       <c r="G45" s="14" t="n">
         <v>123</v>
       </c>
       <c r="H45" s="15" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I45" s="13">
         <f>IF($H$45="","",IF($H$45&lt;0,-$H$45/(-$H$45+100),100/($H$45+100)))</f>
@@ -12593,7 +12593,7 @@
       </c>
       <c r="N45" s="19" t="inlineStr">
         <is>
-          <t>Model 44.8% (fair +123). Your call.</t>
+          <t>Model 44.9% (fair +123). Your call.</t>
         </is>
       </c>
       <c r="O45" s="15" t="n"/>
@@ -12629,7 +12629,7 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.5517098039215687</v>
+        <v>0.5510470588235293</v>
       </c>
       <c r="G46" s="14" t="n">
         <v>-123</v>
@@ -12659,7 +12659,7 @@
       </c>
       <c r="N46" s="19" t="inlineStr">
         <is>
-          <t>Model 55.2% (fair -123). Your call.</t>
+          <t>Model 55.1% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O46" s="15" t="n"/>
@@ -12959,10 +12959,10 @@
         </is>
       </c>
       <c r="F51" s="13" t="n">
-        <v>0.6186806722689074</v>
+        <v>0.6197243697478991</v>
       </c>
       <c r="G51" s="14" t="n">
-        <v>-162</v>
+        <v>-163</v>
       </c>
       <c r="H51" s="15" t="n">
         <v>-138</v>
@@ -12989,7 +12989,7 @@
       </c>
       <c r="N51" s="19" t="inlineStr">
         <is>
-          <t>Model 61.9% (fair -162). Your call.</t>
+          <t>Model 62.0% (fair -163). Your call.</t>
         </is>
       </c>
       <c r="O51" s="15" t="n"/>
@@ -13025,13 +13025,13 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.3813304721030042</v>
+        <v>0.3802978723404255</v>
       </c>
       <c r="G52" s="14" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H52" s="15" t="n">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="I52" s="13">
         <f>IF($H$52="","",IF($H$52&lt;0,-$H$52/(-$H$52+100),100/($H$52+100)))</f>
@@ -13055,7 +13055,7 @@
       </c>
       <c r="N52" s="19" t="inlineStr">
         <is>
-          <t>Model 38.1% (fair +162). Your call.</t>
+          <t>Model 38.0% (fair +163). Your call.</t>
         </is>
       </c>
       <c r="O52" s="15" t="n"/>
@@ -13097,7 +13097,7 @@
         <v>-121</v>
       </c>
       <c r="H53" s="15" t="n">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="I53" s="13">
         <f>IF($H$53="","",IF($H$53&lt;0,-$H$53/(-$H$53+100),100/($H$53+100)))</f>
@@ -13163,7 +13163,7 @@
         <v>121</v>
       </c>
       <c r="H54" s="15" t="n">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="I54" s="13">
         <f>IF($H$54="","",IF($H$54&lt;0,-$H$54/(-$H$54+100),100/($H$54+100)))</f>
@@ -13351,10 +13351,10 @@
         </is>
       </c>
       <c r="F57" s="13" t="n">
-        <v>0.3656</v>
+        <v>0.3676</v>
       </c>
       <c r="G57" s="14" t="n">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H57" s="15" t="n">
         <v>150</v>
@@ -13381,7 +13381,7 @@
       </c>
       <c r="N57" s="19" t="inlineStr">
         <is>
-          <t>Model 36.6% (fair +174). Your call.</t>
+          <t>Model 36.8% (fair +172). Your call.</t>
         </is>
       </c>
       <c r="O57" s="15" t="n"/>
@@ -13417,13 +13417,13 @@
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.6343800000000001</v>
+        <v>0.6324196721311476</v>
       </c>
       <c r="G58" s="14" t="n">
-        <v>-174</v>
+        <v>-172</v>
       </c>
       <c r="H58" s="15" t="n">
-        <v>-150</v>
+        <v>-144</v>
       </c>
       <c r="I58" s="13">
         <f>IF($H$58="","",IF($H$58&lt;0,-$H$58/(-$H$58+100),100/($H$58+100)))</f>
@@ -13447,7 +13447,7 @@
       </c>
       <c r="N58" s="19" t="inlineStr">
         <is>
-          <t>Model 63.4% (fair -174). Your call.</t>
+          <t>Model 63.2% (fair -172). Your call.</t>
         </is>
       </c>
       <c r="O58" s="15" t="n"/>
@@ -13555,7 +13555,7 @@
         <v>167</v>
       </c>
       <c r="H60" s="15" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I60" s="13">
         <f>IF($H$60="","",IF($H$60&lt;0,-$H$60/(-$H$60+100),100/($H$60+100)))</f>
@@ -13621,7 +13621,7 @@
         <v>106</v>
       </c>
       <c r="H61" s="15" t="n">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I61" s="13">
         <f>IF($H$61="","",IF($H$61&lt;0,-$H$61/(-$H$61+100),100/($H$61+100)))</f>
@@ -13687,7 +13687,7 @@
         <v>-106</v>
       </c>
       <c r="H62" s="15" t="n">
-        <v>103</v>
+        <v>-104</v>
       </c>
       <c r="I62" s="13">
         <f>IF($H$62="","",IF($H$62&lt;0,-$H$62/(-$H$62+100),100/($H$62+100)))</f>
@@ -13875,10 +13875,10 @@
         </is>
       </c>
       <c r="F65" s="13" t="n">
-        <v>0.6417</v>
+        <v>0.6282</v>
       </c>
       <c r="G65" s="14" t="n">
-        <v>-179</v>
+        <v>-169</v>
       </c>
       <c r="H65" s="15" t="n"/>
       <c r="I65" s="13">
@@ -13903,7 +13903,7 @@
       </c>
       <c r="N65" s="19" t="inlineStr">
         <is>
-          <t>Model 64.2% (fair -179). Your call.</t>
+          <t>Model 62.8% (fair -169). Your call.</t>
         </is>
       </c>
       <c r="O65" s="15" t="n"/>
@@ -13939,10 +13939,10 @@
         </is>
       </c>
       <c r="F66" s="13" t="n">
-        <v>0.3584</v>
+        <v>0.3718</v>
       </c>
       <c r="G66" s="14" t="n">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="H66" s="15" t="n"/>
       <c r="I66" s="13">
@@ -13967,7 +13967,7 @@
       </c>
       <c r="N66" s="19" t="inlineStr">
         <is>
-          <t>Model 35.8% (fair +179). Your call.</t>
+          <t>Model 37.2% (fair +169). Your call.</t>
         </is>
       </c>
       <c r="O66" s="15" t="n"/>
@@ -14655,13 +14655,13 @@
         </is>
       </c>
       <c r="F77" s="13" t="n">
-        <v>0.3313824884792627</v>
+        <v>0.3285585585585586</v>
       </c>
       <c r="G77" s="14" t="n">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="H77" s="15" t="n">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="I77" s="13">
         <f>IF($H$77="","",IF($H$77&lt;0,-$H$77/(-$H$77+100),100/($H$77+100)))</f>
@@ -14685,7 +14685,7 @@
       </c>
       <c r="N77" s="19" t="inlineStr">
         <is>
-          <t>Model 33.1% (fair +202). Your call.</t>
+          <t>Model 32.9% (fair +204). Your call.</t>
         </is>
       </c>
       <c r="O77" s="15" t="n"/>
@@ -14721,10 +14721,10 @@
         </is>
       </c>
       <c r="F78" s="13" t="n">
-        <v>0.6685819819819819</v>
+        <v>0.6714396396396396</v>
       </c>
       <c r="G78" s="14" t="n">
-        <v>-202</v>
+        <v>-204</v>
       </c>
       <c r="H78" s="15" t="n">
         <v>-122</v>
@@ -14751,7 +14751,7 @@
       </c>
       <c r="N78" s="19" t="inlineStr">
         <is>
-          <t>Model 66.9% (fair -202). Your call.</t>
+          <t>Model 67.1% (fair -204). Your call.</t>
         </is>
       </c>
       <c r="O78" s="15" t="n"/>
@@ -14793,7 +14793,7 @@
         <v>-139</v>
       </c>
       <c r="H79" s="15" t="n">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="I79" s="13">
         <f>IF($H$79="","",IF($H$79&lt;0,-$H$79/(-$H$79+100),100/($H$79+100)))</f>
@@ -15183,13 +15183,13 @@
         </is>
       </c>
       <c r="F85" s="13" t="n">
-        <v>0.5621853658536585</v>
+        <v>0.55175</v>
       </c>
       <c r="G85" s="14" t="n">
-        <v>-128</v>
+        <v>-123</v>
       </c>
       <c r="H85" s="15" t="n">
-        <v>-105</v>
+        <v>100</v>
       </c>
       <c r="I85" s="13">
         <f>IF($H$85="","",IF($H$85&lt;0,-$H$85/(-$H$85+100),100/($H$85+100)))</f>
@@ -15213,7 +15213,7 @@
       </c>
       <c r="N85" s="19" t="inlineStr">
         <is>
-          <t>Model 56.2% (fair -128). Your call.</t>
+          <t>Model 55.2% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O85" s="15" t="n"/>
@@ -15249,13 +15249,13 @@
         </is>
       </c>
       <c r="F86" s="13" t="n">
-        <v>0.43785</v>
+        <v>0.4482333333333333</v>
       </c>
       <c r="G86" s="14" t="n">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="H86" s="15" t="n">
-        <v>100</v>
+        <v>-113</v>
       </c>
       <c r="I86" s="13">
         <f>IF($H$86="","",IF($H$86&lt;0,-$H$86/(-$H$86+100),100/($H$86+100)))</f>
@@ -15279,7 +15279,7 @@
       </c>
       <c r="N86" s="19" t="inlineStr">
         <is>
-          <t>Model 43.8% (fair +128). Your call.</t>
+          <t>Model 44.8% (fair +123). Your call.</t>
         </is>
       </c>
       <c r="O86" s="15" t="n"/>
@@ -15447,10 +15447,10 @@
         </is>
       </c>
       <c r="F89" s="13" t="n">
-        <v>0.5359756756756757</v>
+        <v>0.5276774774774774</v>
       </c>
       <c r="G89" s="14" t="n">
-        <v>-116</v>
+        <v>-112</v>
       </c>
       <c r="H89" s="15" t="n">
         <v>-122</v>
@@ -15477,7 +15477,7 @@
       </c>
       <c r="N89" s="19" t="inlineStr">
         <is>
-          <t>Model 53.6% (fair -116). Your call.</t>
+          <t>Model 52.8% (fair -112). Your call.</t>
         </is>
       </c>
       <c r="O89" s="15" t="n"/>
@@ -15513,10 +15513,10 @@
         </is>
       </c>
       <c r="F90" s="13" t="n">
-        <v>0.4640552995391705</v>
+        <v>0.4723502304147465</v>
       </c>
       <c r="G90" s="14" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="H90" s="15" t="n">
         <v>117</v>
@@ -15543,7 +15543,7 @@
       </c>
       <c r="N90" s="19" t="inlineStr">
         <is>
-          <t>Model 46.4% (fair +115). Your call.</t>
+          <t>Model 47.2% (fair +112). Your call.</t>
         </is>
       </c>
       <c r="O90" s="15" t="n"/>
@@ -15579,10 +15579,10 @@
         </is>
       </c>
       <c r="F91" s="13" t="n">
-        <v>0.6435</v>
+        <v>0.5746</v>
       </c>
       <c r="G91" s="14" t="n">
-        <v>-181</v>
+        <v>-135</v>
       </c>
       <c r="H91" s="15" t="n">
         <v>100</v>
@@ -15609,7 +15609,7 @@
       </c>
       <c r="N91" s="19" t="inlineStr">
         <is>
-          <t>Model 64.3% (fair -181). Your call.</t>
+          <t>Model 57.5% (fair -135). Your call.</t>
         </is>
       </c>
       <c r="O91" s="15" t="n"/>
@@ -15645,13 +15645,13 @@
         </is>
       </c>
       <c r="F92" s="13" t="n">
-        <v>0.3565</v>
+        <v>0.4253658536585366</v>
       </c>
       <c r="G92" s="14" t="n">
-        <v>181</v>
+        <v>135</v>
       </c>
       <c r="H92" s="15" t="n">
-        <v>245</v>
+        <v>105</v>
       </c>
       <c r="I92" s="13">
         <f>IF($H$92="","",IF($H$92&lt;0,-$H$92/(-$H$92+100),100/($H$92+100)))</f>
@@ -15675,7 +15675,7 @@
       </c>
       <c r="N92" s="19" t="inlineStr">
         <is>
-          <t>Model 35.7% (fair +181). Your call.</t>
+          <t>Model 42.5% (fair +135). Your call.</t>
         </is>
       </c>
       <c r="O92" s="15" t="n"/>
@@ -15711,10 +15711,10 @@
         </is>
       </c>
       <c r="F93" s="13" t="n">
-        <v>0.6226745098039216</v>
+        <v>0.6312450980392157</v>
       </c>
       <c r="G93" s="14" t="n">
-        <v>-165</v>
+        <v>-171</v>
       </c>
       <c r="H93" s="15" t="n">
         <v>-155</v>
@@ -15741,7 +15741,7 @@
       </c>
       <c r="N93" s="19" t="inlineStr">
         <is>
-          <t>Model 62.3% (fair -165). Your call.</t>
+          <t>Model 63.1% (fair -171). Your call.</t>
         </is>
       </c>
       <c r="O93" s="15" t="n"/>
@@ -15777,10 +15777,10 @@
         </is>
       </c>
       <c r="F94" s="13" t="n">
-        <v>0.3773333333333334</v>
+        <v>0.3687916666666667</v>
       </c>
       <c r="G94" s="14" t="n">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="H94" s="15" t="n">
         <v>140</v>
@@ -15807,7 +15807,7 @@
       </c>
       <c r="N94" s="19" t="inlineStr">
         <is>
-          <t>Model 37.7% (fair +165). Your call.</t>
+          <t>Model 36.9% (fair +171). Your call.</t>
         </is>
       </c>
       <c r="O94" s="15" t="n"/>
@@ -15843,13 +15843,13 @@
         </is>
       </c>
       <c r="F95" s="13" t="n">
-        <v>0.54865</v>
+        <v>0.54375</v>
       </c>
       <c r="G95" s="14" t="n">
-        <v>-122</v>
+        <v>-119</v>
       </c>
       <c r="H95" s="15" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="I95" s="13">
         <f>IF($H$95="","",IF($H$95&lt;0,-$H$95/(-$H$95+100),100/($H$95+100)))</f>
@@ -15873,7 +15873,7 @@
       </c>
       <c r="N95" s="19" t="inlineStr">
         <is>
-          <t>Model 54.9% (fair -122). Your call.</t>
+          <t>Model 54.4% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O95" s="15" t="n"/>
@@ -15909,10 +15909,10 @@
         </is>
       </c>
       <c r="F96" s="13" t="n">
-        <v>0.45135</v>
+        <v>0.45625</v>
       </c>
       <c r="G96" s="14" t="n">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="H96" s="15" t="n">
         <v>100</v>
@@ -15939,7 +15939,7 @@
       </c>
       <c r="N96" s="19" t="inlineStr">
         <is>
-          <t>Model 45.1% (fair +122). Your call.</t>
+          <t>Model 45.6% (fair +119). Your call.</t>
         </is>
       </c>
       <c r="O96" s="15" t="n"/>
@@ -15975,13 +15975,13 @@
         </is>
       </c>
       <c r="F97" s="13" t="n">
-        <v>0.49165</v>
+        <v>0.4867788461538461</v>
       </c>
       <c r="G97" s="14" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H97" s="15" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="I97" s="13">
         <f>IF($H$97="","",IF($H$97&lt;0,-$H$97/(-$H$97+100),100/($H$97+100)))</f>
@@ -16005,7 +16005,7 @@
       </c>
       <c r="N97" s="19" t="inlineStr">
         <is>
-          <t>Model 49.2% (fair +103). Your call.</t>
+          <t>Model 48.7% (fair +105). Your call.</t>
         </is>
       </c>
       <c r="O97" s="15" t="n"/>
@@ -16041,10 +16041,10 @@
         </is>
       </c>
       <c r="F98" s="13" t="n">
-        <v>0.50835</v>
+        <v>0.51325</v>
       </c>
       <c r="G98" s="14" t="n">
-        <v>-103</v>
+        <v>-105</v>
       </c>
       <c r="H98" s="15" t="n">
         <v>100</v>
@@ -16071,7 +16071,7 @@
       </c>
       <c r="N98" s="19" t="inlineStr">
         <is>
-          <t>Model 50.8% (fair -103). Your call.</t>
+          <t>Model 51.3% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O98" s="15" t="n"/>
@@ -16899,10 +16899,10 @@
         </is>
       </c>
       <c r="F111" s="13" t="n">
-        <v>0.52885</v>
+        <v>0.53585</v>
       </c>
       <c r="G111" s="14" t="n">
-        <v>-112</v>
+        <v>-115</v>
       </c>
       <c r="H111" s="15" t="n">
         <v>100</v>
@@ -16929,7 +16929,7 @@
       </c>
       <c r="N111" s="19" t="inlineStr">
         <is>
-          <t>Model 52.9% (fair -112). Your call.</t>
+          <t>Model 53.6% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O111" s="15" t="n"/>
@@ -16965,13 +16965,13 @@
         </is>
       </c>
       <c r="F112" s="13" t="n">
-        <v>0.4711271889400921</v>
+        <v>0.4641764705882352</v>
       </c>
       <c r="G112" s="14" t="n">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="H112" s="15" t="n">
-        <v>-117</v>
+        <v>-104</v>
       </c>
       <c r="I112" s="13">
         <f>IF($H$112="","",IF($H$112&lt;0,-$H$112/(-$H$112+100),100/($H$112+100)))</f>
@@ -16995,7 +16995,7 @@
       </c>
       <c r="N112" s="19" t="inlineStr">
         <is>
-          <t>Model 47.1% (fair +112). Your call.</t>
+          <t>Model 46.4% (fair +115). Your call.</t>
         </is>
       </c>
       <c r="O112" s="15" t="n"/>
@@ -17295,10 +17295,10 @@
         </is>
       </c>
       <c r="F117" s="13" t="n">
-        <v>0.5817512195121951</v>
+        <v>0.5866682926829269</v>
       </c>
       <c r="G117" s="14" t="n">
-        <v>-139</v>
+        <v>-142</v>
       </c>
       <c r="H117" s="15" t="n">
         <v>-105</v>
@@ -17325,7 +17325,7 @@
       </c>
       <c r="N117" s="19" t="inlineStr">
         <is>
-          <t>Model 58.2% (fair -139). Your call.</t>
+          <t>Model 58.7% (fair -142). Your call.</t>
         </is>
       </c>
       <c r="O117" s="15" t="n"/>
@@ -17361,13 +17361,13 @@
         </is>
       </c>
       <c r="F118" s="13" t="n">
-        <v>0.41825</v>
+        <v>0.4133173076923077</v>
       </c>
       <c r="G118" s="14" t="n">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="H118" s="15" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="I118" s="13">
         <f>IF($H$118="","",IF($H$118&lt;0,-$H$118/(-$H$118+100),100/($H$118+100)))</f>
@@ -17391,7 +17391,7 @@
       </c>
       <c r="N118" s="19" t="inlineStr">
         <is>
-          <t>Model 41.8% (fair +139). Your call.</t>
+          <t>Model 41.3% (fair +142). Your call.</t>
         </is>
       </c>
       <c r="O118" s="15" t="n"/>
@@ -18075,10 +18075,10 @@
         </is>
       </c>
       <c r="F129" s="13" t="n">
-        <v>0.5612634146341464</v>
+        <v>0.5636707317073171</v>
       </c>
       <c r="G129" s="14" t="n">
-        <v>-128</v>
+        <v>-129</v>
       </c>
       <c r="H129" s="15" t="n">
         <v>-105</v>
@@ -18105,7 +18105,7 @@
       </c>
       <c r="N129" s="19" t="inlineStr">
         <is>
-          <t>Model 56.1% (fair -128). Your call.</t>
+          <t>Model 56.4% (fair -129). Your call.</t>
         </is>
       </c>
       <c r="O129" s="15" t="n"/>
@@ -18141,13 +18141,13 @@
         </is>
       </c>
       <c r="F130" s="13" t="n">
-        <v>0.4387254901960784</v>
+        <v>0.4362980769230769</v>
       </c>
       <c r="G130" s="14" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H130" s="15" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I130" s="13">
         <f>IF($H$130="","",IF($H$130&lt;0,-$H$130/(-$H$130+100),100/($H$130+100)))</f>
@@ -18171,7 +18171,7 @@
       </c>
       <c r="N130" s="19" t="inlineStr">
         <is>
-          <t>Model 43.9% (fair +128). Your call.</t>
+          <t>Model 43.6% (fair +129). Your call.</t>
         </is>
       </c>
       <c r="O130" s="15" t="n"/>
@@ -18473,7 +18473,7 @@
         <v>113</v>
       </c>
       <c r="H135" s="15" t="n">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="I135" s="13">
         <f>IF($H$135="","",IF($H$135&lt;0,-$H$135/(-$H$135+100),100/($H$135+100)))</f>
@@ -18731,10 +18731,10 @@
         </is>
       </c>
       <c r="F139" s="13" t="n">
-        <v>0.5516</v>
+        <v>0.5442</v>
       </c>
       <c r="G139" s="14" t="n">
-        <v>-123</v>
+        <v>-119</v>
       </c>
       <c r="H139" s="15" t="n"/>
       <c r="I139" s="13">
@@ -18759,7 +18759,7 @@
       </c>
       <c r="N139" s="19" t="inlineStr">
         <is>
-          <t>Model 55.2% (fair -123). Your call.</t>
+          <t>Model 54.4% (fair -119). Your call.</t>
         </is>
       </c>
       <c r="O139" s="15" t="n"/>
@@ -18795,10 +18795,10 @@
         </is>
       </c>
       <c r="F140" s="13" t="n">
-        <v>0.4484162995594714</v>
+        <v>0.4558013215859031</v>
       </c>
       <c r="G140" s="14" t="n">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="H140" s="15" t="n">
         <v>-127</v>
@@ -18825,7 +18825,7 @@
       </c>
       <c r="N140" s="19" t="inlineStr">
         <is>
-          <t>Model 44.8% (fair +123). Your call.</t>
+          <t>Model 45.6% (fair +119). Your call.</t>
         </is>
       </c>
       <c r="O140" s="15" t="n"/>
@@ -18861,10 +18861,10 @@
         </is>
       </c>
       <c r="F141" s="13" t="n">
-        <v>0.4769048780487805</v>
+        <v>0.4827439024390244</v>
       </c>
       <c r="G141" s="14" t="n">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="H141" s="15" t="n">
         <v>-105</v>
@@ -18891,7 +18891,7 @@
       </c>
       <c r="N141" s="19" t="inlineStr">
         <is>
-          <t>Model 47.7% (fair +110). Your call.</t>
+          <t>Model 48.3% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O141" s="15" t="n"/>
@@ -18927,13 +18927,13 @@
         </is>
       </c>
       <c r="F142" s="13" t="n">
-        <v>0.5231</v>
+        <v>0.5172596153846154</v>
       </c>
       <c r="G142" s="14" t="n">
-        <v>-110</v>
+        <v>-107</v>
       </c>
       <c r="H142" s="15" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="I142" s="13">
         <f>IF($H$142="","",IF($H$142&lt;0,-$H$142/(-$H$142+100),100/($H$142+100)))</f>
@@ -18957,7 +18957,7 @@
       </c>
       <c r="N142" s="19" t="inlineStr">
         <is>
-          <t>Model 52.3% (fair -110). Your call.</t>
+          <t>Model 51.7% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O142" s="15" t="n"/>
@@ -18993,10 +18993,10 @@
         </is>
       </c>
       <c r="F143" s="13" t="n">
-        <v>0.2763921568627451</v>
+        <v>0.2867058823529413</v>
       </c>
       <c r="G143" s="14" t="n">
-        <v>262</v>
+        <v>249</v>
       </c>
       <c r="H143" s="15" t="n">
         <v>155</v>
@@ -19023,7 +19023,7 @@
       </c>
       <c r="N143" s="19" t="inlineStr">
         <is>
-          <t>Model 27.6% (fair +262). Your call.</t>
+          <t>Model 28.7% (fair +249). Your call.</t>
         </is>
       </c>
       <c r="O143" s="15" t="n"/>
@@ -19059,10 +19059,10 @@
         </is>
       </c>
       <c r="F144" s="13" t="n">
-        <v>0.7236</v>
+        <v>0.7133</v>
       </c>
       <c r="G144" s="14" t="n">
-        <v>-262</v>
+        <v>-249</v>
       </c>
       <c r="H144" s="15" t="n"/>
       <c r="I144" s="13">
@@ -19087,7 +19087,7 @@
       </c>
       <c r="N144" s="19" t="inlineStr">
         <is>
-          <t>Model 72.4% (fair -262). Your call.</t>
+          <t>Model 71.3% (fair -249). Your call.</t>
         </is>
       </c>
       <c r="O144" s="15" t="n"/>
@@ -19120,7 +19120,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P46"/>
+  <dimension ref="A1:P40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -19245,12 +19245,12 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Phoenix Mercury @ Toronto Tempo</t>
+          <t>Los Angeles Sparks @ Indiana Fever</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
@@ -19260,17 +19260,17 @@
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Phoenix Mercury</t>
+          <t>Los Angeles Sparks</t>
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.3492079207920792</v>
+        <v>0.2905507246376811</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>186</v>
+        <v>244</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>203</v>
+        <v>245</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -19294,7 +19294,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 34.9% (fair +186). Your call.</t>
+          <t>Model 29.1% (fair +244). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -19311,12 +19311,12 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Phoenix Mercury @ Toronto Tempo</t>
+          <t>Los Angeles Sparks @ Indiana Fever</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
@@ -19326,17 +19326,17 @@
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Toronto Tempo</t>
+          <t>Indiana Fever</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.6508238095238095</v>
+        <v>0.7094504273504273</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-186</v>
+        <v>-244</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-194</v>
+        <v>-251</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -19360,7 +19360,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 65.1% (fair -186). Your call.</t>
+          <t>Model 70.9% (fair -244). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -19377,12 +19377,12 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Phoenix Mercury @ Toronto Tempo</t>
+          <t>Los Angeles Sparks @ Indiana Fever</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -19396,13 +19396,13 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.6043749999999999</v>
+        <v>0.715</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-153</v>
+        <v>-251</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>108</v>
+        <v>-104</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -19426,7 +19426,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 60.4% (fair -153). Your call.</t>
+          <t>Model 71.5% (fair -251). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -19443,12 +19443,12 @@
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Phoenix Mercury @ Toronto Tempo</t>
+          <t>Los Angeles Sparks @ Indiana Fever</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
@@ -19462,13 +19462,13 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.3956</v>
+        <v>0.285</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>153</v>
+        <v>251</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>108</v>
+        <v>-104</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -19492,7 +19492,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 39.6% (fair +153). Your call.</t>
+          <t>Model 28.5% (fair +251). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -19509,12 +19509,12 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Phoenix Mercury @ Toronto Tempo</t>
+          <t>Los Angeles Sparks @ Indiana Fever</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -19524,17 +19524,17 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Toronto Tempo -6.5</t>
+          <t>Indiana Fever -6.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.4702</v>
+        <v>0.513</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>113</v>
+        <v>-105</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>113</v>
+        <v>-108</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -19558,7 +19558,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 47.0% (fair +113). Your call.</t>
+          <t>Model 51.3% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -19575,12 +19575,12 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Phoenix Mercury @ Toronto Tempo</t>
+          <t>Los Angeles Sparks @ Indiana Fever</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
@@ -19590,17 +19590,17 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Phoenix Mercury +6.5</t>
+          <t>Los Angeles Sparks +6.5</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5298</v>
+        <v>0.4869756097560976</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-113</v>
+        <v>105</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -19624,7 +19624,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 53.0% (fair -113). Your call.</t>
+          <t>Model 48.7% (fair +105). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -19641,12 +19641,12 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Indiana Fever</t>
+          <t>Atlanta Dream @ Seattle Storm</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:00</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -19656,17 +19656,17 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks</t>
+          <t>Atlanta Dream</t>
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.2901159420289854</v>
+        <v>0.7612197530864198</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>245</v>
+        <v>-319</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>245</v>
+        <v>-305</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -19690,7 +19690,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 29.0% (fair +245). Your call.</t>
+          <t>Model 76.1% (fair -319). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -19707,12 +19707,12 @@
       </c>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Indiana Fever</t>
+          <t>Atlanta Dream @ Seattle Storm</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:00</t>
         </is>
       </c>
       <c r="D12" s="20" t="inlineStr">
@@ -19722,17 +19722,17 @@
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
-          <t>Indiana Fever</t>
+          <t>Seattle Storm</t>
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.7099056338028169</v>
+        <v>0.238825</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-245</v>
+        <v>319</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>-255</v>
+        <v>300</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -19756,7 +19756,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 71.0% (fair -245). Your call.</t>
+          <t>Model 23.9% (fair +319). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -19773,12 +19773,12 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Indiana Fever</t>
+          <t>Atlanta Dream @ Seattle Storm</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:00</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
@@ -19792,13 +19792,13 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.715</v>
+        <v>0.2606730769230769</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-251</v>
+        <v>284</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>-104</v>
+        <v>108</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -19822,7 +19822,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 71.5% (fair -251). Your call.</t>
+          <t>Model 26.1% (fair +284). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -19839,12 +19839,12 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Indiana Fever</t>
+          <t>Atlanta Dream @ Seattle Storm</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:00</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
@@ -19858,13 +19858,13 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.285</v>
+        <v>0.7393000000000001</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>251</v>
+        <v>-284</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>-104</v>
+        <v>108</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -19888,7 +19888,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 28.5% (fair +251). Your call.</t>
+          <t>Model 73.9% (fair -284). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -19905,12 +19905,12 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Indiana Fever</t>
+          <t>Atlanta Dream @ Seattle Storm</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:00</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -19920,17 +19920,17 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Indiana Fever -6.5</t>
+          <t>Seattle Storm -4.5</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.510709756097561</v>
+        <v>0.1855</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-104</v>
+        <v>439</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>-105</v>
+        <v>410</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -19954,7 +19954,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 51.1% (fair -104). Your call.</t>
+          <t>Model 18.6% (fair +439). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -19971,12 +19971,12 @@
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Indiana Fever</t>
+          <t>Atlanta Dream @ Seattle Storm</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:00</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
@@ -19986,17 +19986,17 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks +6.5</t>
+          <t>Atlanta Dream +4.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.4893137254901961</v>
+        <v>0.8145</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>104</v>
+        <v>-439</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -20020,7 +20020,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 48.9% (fair +104). Your call.</t>
+          <t>Model 81.5% (fair -439). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -20032,17 +20032,17 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Atlanta Dream @ Seattle Storm</t>
+          <t>Minnesota Lynx @ Dallas Wings</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>01:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -20052,17 +20052,17 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Atlanta Dream</t>
+          <t>Minnesota Lynx</t>
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.7608</v>
+        <v>0.6274734375000001</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-318</v>
+        <v>-168</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>-300</v>
+        <v>-156</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -20086,7 +20086,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 76.1% (fair -318). Your call.</t>
+          <t>Model 62.7% (fair -168). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -20098,17 +20098,17 @@
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>Atlanta Dream @ Seattle Storm</t>
+          <t>Minnesota Lynx @ Dallas Wings</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>01:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
@@ -20118,17 +20118,17 @@
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>Seattle Storm</t>
+          <t>Dallas Wings</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.2392</v>
+        <v>0.3725095057034221</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>318</v>
+        <v>168</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>300</v>
+        <v>163</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -20152,7 +20152,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 23.9% (fair +318). Your call.</t>
+          <t>Model 37.3% (fair +168). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -20164,17 +20164,17 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Atlanta Dream @ Seattle Storm</t>
+          <t>Minnesota Lynx @ Dallas Wings</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>01:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -20184,17 +20184,17 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Over 179.5</t>
+          <t>Over 177.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.2606730769230769</v>
+        <v>0.4101</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>284</v>
+        <v>144</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -20218,7 +20218,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 26.1% (fair +284). Your call.</t>
+          <t>Model 41.0% (fair +144). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -20230,17 +20230,17 @@
     <row r="20">
       <c r="A20" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>Atlanta Dream @ Seattle Storm</t>
+          <t>Minnesota Lynx @ Dallas Wings</t>
         </is>
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
-          <t>01:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
@@ -20250,17 +20250,17 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Under 179.5</t>
+          <t>Under 177.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.7393000000000001</v>
+        <v>0.5899</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>-284</v>
+        <v>-144</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -20284,7 +20284,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 73.9% (fair -284). Your call.</t>
+          <t>Model 59.0% (fair -144). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -20296,17 +20296,17 @@
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>Atlanta Dream @ Seattle Storm</t>
+          <t>Minnesota Lynx @ Dallas Wings</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>01:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
@@ -20316,17 +20316,17 @@
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Seattle Storm -4.5</t>
+          <t>Dallas Wings +3.5</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.1855</v>
+        <v>0.5042</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>439</v>
+        <v>-102</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>430</v>
+        <v>113</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -20350,7 +20350,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 18.6% (fair +439). Your call.</t>
+          <t>Model 50.4% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -20362,17 +20362,17 @@
     <row r="22">
       <c r="A22" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>Atlanta Dream @ Seattle Storm</t>
+          <t>Minnesota Lynx @ Dallas Wings</t>
         </is>
       </c>
       <c r="C22" s="20" t="inlineStr">
         <is>
-          <t>01:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D22" s="20" t="inlineStr">
@@ -20382,14 +20382,14 @@
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Atlanta Dream +4.5</t>
+          <t>Minnesota Lynx -3.5</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.8145</v>
+        <v>0.4958</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-439</v>
+        <v>102</v>
       </c>
       <c r="H22" s="15" t="n">
         <v>108</v>
@@ -20416,7 +20416,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 81.5% (fair -439). Your call.</t>
+          <t>Model 49.6% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -20433,12 +20433,12 @@
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>Minnesota Lynx @ Dallas Wings</t>
+          <t>Portland Fire @ Washington Mystics</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
@@ -20448,17 +20448,17 @@
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Minnesota Lynx</t>
+          <t>Portland Fire</t>
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.6243046875</v>
+        <v>0.3029129129129129</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>-166</v>
+        <v>230</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>-156</v>
+        <v>233</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -20482,7 +20482,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 62.4% (fair -166). Your call.</t>
+          <t>Model 30.3% (fair +230). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -20499,12 +20499,12 @@
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>Minnesota Lynx @ Dallas Wings</t>
+          <t>Portland Fire @ Washington Mystics</t>
         </is>
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
@@ -20514,17 +20514,17 @@
       </c>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>Dallas Wings</t>
+          <t>Washington Mystics</t>
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.375703125</v>
+        <v>0.6970782608695653</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>166</v>
+        <v>-230</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>156</v>
+        <v>-245</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -20548,7 +20548,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 37.6% (fair +166). Your call.</t>
+          <t>Model 69.7% (fair -230). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -20565,12 +20565,12 @@
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Minnesota Lynx @ Dallas Wings</t>
+          <t>Portland Fire @ Washington Mystics</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
@@ -20580,17 +20580,17 @@
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Over 177.5</t>
+          <t>Over 166.5</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.4101</v>
+        <v>0.5774509803921568</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>144</v>
+        <v>-137</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -20614,7 +20614,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 41.0% (fair +144). Your call.</t>
+          <t>Model 57.7% (fair -137). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -20631,12 +20631,12 @@
       </c>
       <c r="B26" s="20" t="inlineStr">
         <is>
-          <t>Minnesota Lynx @ Dallas Wings</t>
+          <t>Portland Fire @ Washington Mystics</t>
         </is>
       </c>
       <c r="C26" s="20" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D26" s="20" t="inlineStr">
@@ -20646,17 +20646,17 @@
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Under 177.5</t>
+          <t>Under 166.5</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.5899</v>
+        <v>0.4226</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>-144</v>
+        <v>137</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -20680,7 +20680,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 59.0% (fair -144). Your call.</t>
+          <t>Model 42.3% (fair +137). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -20697,12 +20697,12 @@
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>Minnesota Lynx @ Dallas Wings</t>
+          <t>Portland Fire @ Washington Mystics</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
@@ -20712,17 +20712,17 @@
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Dallas Wings +3.5</t>
+          <t>Washington Mystics -6.5</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.5042</v>
+        <v>0.47875</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>-102</v>
+        <v>109</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -20746,7 +20746,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 50.4% (fair -102). Your call.</t>
+          <t>Model 47.9% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -20763,12 +20763,12 @@
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>Minnesota Lynx @ Dallas Wings</t>
+          <t>Portland Fire @ Washington Mystics</t>
         </is>
       </c>
       <c r="C28" s="20" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
@@ -20778,17 +20778,17 @@
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>Minnesota Lynx -3.5</t>
+          <t>Portland Fire +6.5</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.4958</v>
+        <v>0.5212376237623763</v>
       </c>
       <c r="G28" s="14" t="n">
+        <v>-109</v>
+      </c>
+      <c r="H28" s="15" t="n">
         <v>102</v>
-      </c>
-      <c r="H28" s="15" t="n">
-        <v>104</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -20812,7 +20812,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 49.6% (fair +102). Your call.</t>
+          <t>Model 52.1% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -20829,12 +20829,12 @@
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>Portland Fire @ Washington Mystics</t>
+          <t>Las Vegas Aces @ Chicago Sky</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
@@ -20844,17 +20844,17 @@
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>Portland Fire</t>
+          <t>Las Vegas Aces</t>
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.3017117117117117</v>
+        <v>0.7520298701298702</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>231</v>
+        <v>-303</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>233</v>
+        <v>-285</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -20878,7 +20878,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 30.2% (fair +231). Your call.</t>
+          <t>Model 75.2% (fair -303). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -20895,12 +20895,12 @@
       </c>
       <c r="B30" s="20" t="inlineStr">
         <is>
-          <t>Portland Fire @ Washington Mystics</t>
+          <t>Las Vegas Aces @ Chicago Sky</t>
         </is>
       </c>
       <c r="C30" s="20" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D30" s="20" t="inlineStr">
@@ -20910,17 +20910,17 @@
       </c>
       <c r="E30" s="20" t="inlineStr">
         <is>
-          <t>Washington Mystics</t>
+          <t>Chicago Sky</t>
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.698269014084507</v>
+        <v>0.247975</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-231</v>
+        <v>303</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>-255</v>
+        <v>300</v>
       </c>
       <c r="I30" s="13">
         <f>IF($H$30="","",IF($H$30&lt;0,-$H$30/(-$H$30+100),100/($H$30+100)))</f>
@@ -20944,7 +20944,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Model 69.8% (fair -231). Your call.</t>
+          <t>Model 24.8% (fair +303). Your call.</t>
         </is>
       </c>
       <c r="O30" s="15" t="n"/>
@@ -20961,12 +20961,12 @@
       </c>
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>Portland Fire @ Washington Mystics</t>
+          <t>Las Vegas Aces @ Chicago Sky</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D31" s="12" t="inlineStr">
@@ -20976,14 +20976,14 @@
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>Over 165.5</t>
+          <t>Over 178.5</t>
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.6033500000000001</v>
+        <v>0.55275</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>-152</v>
+        <v>-124</v>
       </c>
       <c r="H31" s="15" t="n">
         <v>100</v>
@@ -21010,7 +21010,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 60.3% (fair -152). Your call.</t>
+          <t>Model 55.3% (fair -124). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -21027,12 +21027,12 @@
       </c>
       <c r="B32" s="20" t="inlineStr">
         <is>
-          <t>Portland Fire @ Washington Mystics</t>
+          <t>Las Vegas Aces @ Chicago Sky</t>
         </is>
       </c>
       <c r="C32" s="20" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D32" s="20" t="inlineStr">
@@ -21042,14 +21042,14 @@
       </c>
       <c r="E32" s="20" t="inlineStr">
         <is>
-          <t>Under 165.5</t>
+          <t>Under 178.5</t>
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.3967000000000001</v>
+        <v>0.4472</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>152</v>
+        <v>124</v>
       </c>
       <c r="H32" s="15" t="n">
         <v>100</v>
@@ -21076,7 +21076,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 39.7% (fair +152). Your call.</t>
+          <t>Model 44.7% (fair +124). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -21093,12 +21093,12 @@
       </c>
       <c r="B33" s="12" t="inlineStr">
         <is>
-          <t>Portland Fire @ Washington Mystics</t>
+          <t>Las Vegas Aces @ Chicago Sky</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D33" s="12" t="inlineStr">
@@ -21108,17 +21108,17 @@
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>Washington Mystics -6.5</t>
+          <t>Chicago Sky +7.5</t>
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.4811529411764706</v>
+        <v>0.5767615384615384</v>
       </c>
       <c r="G33" s="14" t="n">
-        <v>108</v>
+        <v>-136</v>
       </c>
       <c r="H33" s="15" t="n">
-        <v>-104</v>
+        <v>-108</v>
       </c>
       <c r="I33" s="13">
         <f>IF($H$33="","",IF($H$33&lt;0,-$H$33/(-$H$33+100),100/($H$33+100)))</f>
@@ -21142,7 +21142,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>Model 48.1% (fair +108). Your call.</t>
+          <t>Model 57.7% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O33" s="15" t="n"/>
@@ -21159,12 +21159,12 @@
       </c>
       <c r="B34" s="20" t="inlineStr">
         <is>
-          <t>Portland Fire @ Washington Mystics</t>
+          <t>Las Vegas Aces @ Chicago Sky</t>
         </is>
       </c>
       <c r="C34" s="20" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D34" s="20" t="inlineStr">
@@ -21174,17 +21174,17 @@
       </c>
       <c r="E34" s="20" t="inlineStr">
         <is>
-          <t>Portland Fire +6.5</t>
+          <t>Las Vegas Aces -7.5</t>
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.5188118811881188</v>
+        <v>0.4232380952380952</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>-108</v>
+        <v>136</v>
       </c>
       <c r="H34" s="15" t="n">
-        <v>102</v>
+        <v>-110</v>
       </c>
       <c r="I34" s="13">
         <f>IF($H$34="","",IF($H$34&lt;0,-$H$34/(-$H$34+100),100/($H$34+100)))</f>
@@ -21208,7 +21208,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>Model 51.9% (fair -108). Your call.</t>
+          <t>Model 42.3% (fair +136). Your call.</t>
         </is>
       </c>
       <c r="O34" s="15" t="n"/>
@@ -21225,12 +21225,12 @@
       </c>
       <c r="B35" s="12" t="inlineStr">
         <is>
-          <t>Las Vegas Aces @ Chicago Sky</t>
+          <t>New York Liberty @ Golden State Valkyries</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D35" s="12" t="inlineStr">
@@ -21240,17 +21240,17 @@
       </c>
       <c r="E35" s="12" t="inlineStr">
         <is>
-          <t>Las Vegas Aces</t>
+          <t>New York Liberty</t>
         </is>
       </c>
       <c r="F35" s="13" t="n">
-        <v>0.7489948979591837</v>
+        <v>0.4216826923076923</v>
       </c>
       <c r="G35" s="14" t="n">
-        <v>-298</v>
+        <v>137</v>
       </c>
       <c r="H35" s="15" t="n">
-        <v>-292</v>
+        <v>108</v>
       </c>
       <c r="I35" s="13">
         <f>IF($H$35="","",IF($H$35&lt;0,-$H$35/(-$H$35+100),100/($H$35+100)))</f>
@@ -21274,7 +21274,7 @@
       </c>
       <c r="N35" s="19" t="inlineStr">
         <is>
-          <t>Model 74.9% (fair -298). Your call.</t>
+          <t>Model 42.2% (fair +137). Your call.</t>
         </is>
       </c>
       <c r="O35" s="15" t="n"/>
@@ -21291,12 +21291,12 @@
       </c>
       <c r="B36" s="20" t="inlineStr">
         <is>
-          <t>Las Vegas Aces @ Chicago Sky</t>
+          <t>New York Liberty @ Golden State Valkyries</t>
         </is>
       </c>
       <c r="C36" s="20" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D36" s="20" t="inlineStr">
@@ -21306,17 +21306,17 @@
       </c>
       <c r="E36" s="20" t="inlineStr">
         <is>
-          <t>Chicago Sky</t>
+          <t>Golden State Valkyries</t>
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.251012987012987</v>
+        <v>0.578321568627451</v>
       </c>
       <c r="G36" s="14" t="n">
-        <v>298</v>
+        <v>-137</v>
       </c>
       <c r="H36" s="15" t="n">
-        <v>285</v>
+        <v>-104</v>
       </c>
       <c r="I36" s="13">
         <f>IF($H$36="","",IF($H$36&lt;0,-$H$36/(-$H$36+100),100/($H$36+100)))</f>
@@ -21340,7 +21340,7 @@
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>Model 25.1% (fair +298). Your call.</t>
+          <t>Model 57.8% (fair -137). Your call.</t>
         </is>
       </c>
       <c r="O36" s="15" t="n"/>
@@ -21357,12 +21357,12 @@
       </c>
       <c r="B37" s="12" t="inlineStr">
         <is>
-          <t>Las Vegas Aces @ Chicago Sky</t>
+          <t>New York Liberty @ Golden State Valkyries</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D37" s="12" t="inlineStr">
@@ -21372,17 +21372,17 @@
       </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>Over 178.5</t>
+          <t>Over 163.5</t>
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>0.55275</v>
+        <v>0.5769238095238095</v>
       </c>
       <c r="G37" s="14" t="n">
-        <v>-124</v>
+        <v>-136</v>
       </c>
       <c r="H37" s="15" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="I37" s="13">
         <f>IF($H$37="","",IF($H$37&lt;0,-$H$37/(-$H$37+100),100/($H$37+100)))</f>
@@ -21406,7 +21406,7 @@
       </c>
       <c r="N37" s="19" t="inlineStr">
         <is>
-          <t>Model 55.3% (fair -124). Your call.</t>
+          <t>Model 57.7% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O37" s="15" t="n"/>
@@ -21423,12 +21423,12 @@
       </c>
       <c r="B38" s="20" t="inlineStr">
         <is>
-          <t>Las Vegas Aces @ Chicago Sky</t>
+          <t>New York Liberty @ Golden State Valkyries</t>
         </is>
       </c>
       <c r="C38" s="20" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D38" s="20" t="inlineStr">
@@ -21438,17 +21438,17 @@
       </c>
       <c r="E38" s="20" t="inlineStr">
         <is>
-          <t>Under 178.5</t>
+          <t>Under 163.5</t>
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.4472</v>
+        <v>0.4231</v>
       </c>
       <c r="G38" s="14" t="n">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="H38" s="15" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="I38" s="13">
         <f>IF($H$38="","",IF($H$38&lt;0,-$H$38/(-$H$38+100),100/($H$38+100)))</f>
@@ -21472,7 +21472,7 @@
       </c>
       <c r="N38" s="19" t="inlineStr">
         <is>
-          <t>Model 44.7% (fair +124). Your call.</t>
+          <t>Model 42.3% (fair +136). Your call.</t>
         </is>
       </c>
       <c r="O38" s="15" t="n"/>
@@ -21489,12 +21489,12 @@
       </c>
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>Las Vegas Aces @ Chicago Sky</t>
+          <t>New York Liberty @ Golden State Valkyries</t>
         </is>
       </c>
       <c r="C39" s="12" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D39" s="12" t="inlineStr">
@@ -21504,17 +21504,17 @@
       </c>
       <c r="E39" s="12" t="inlineStr">
         <is>
-          <t>Chicago Sky +7.5</t>
+          <t>Golden State Valkyries +1.5</t>
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>0.5767615384615384</v>
+        <v>0.5795450980392156</v>
       </c>
       <c r="G39" s="14" t="n">
-        <v>-136</v>
+        <v>-138</v>
       </c>
       <c r="H39" s="15" t="n">
-        <v>-108</v>
+        <v>-104</v>
       </c>
       <c r="I39" s="13">
         <f>IF($H$39="","",IF($H$39&lt;0,-$H$39/(-$H$39+100),100/($H$39+100)))</f>
@@ -21538,7 +21538,7 @@
       </c>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -136). Your call.</t>
+          <t>Model 58.0% (fair -138). Your call.</t>
         </is>
       </c>
       <c r="O39" s="15" t="n"/>
@@ -21555,12 +21555,12 @@
       </c>
       <c r="B40" s="20" t="inlineStr">
         <is>
-          <t>Las Vegas Aces @ Chicago Sky</t>
+          <t>New York Liberty @ Golden State Valkyries</t>
         </is>
       </c>
       <c r="C40" s="20" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D40" s="20" t="inlineStr">
@@ -21570,17 +21570,17 @@
       </c>
       <c r="E40" s="20" t="inlineStr">
         <is>
-          <t>Las Vegas Aces -7.5</t>
+          <t>New York Liberty -1.5</t>
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.4232380952380952</v>
+        <v>0.4204878048780488</v>
       </c>
       <c r="G40" s="14" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H40" s="15" t="n">
-        <v>-110</v>
+        <v>105</v>
       </c>
       <c r="I40" s="13">
         <f>IF($H$40="","",IF($H$40&lt;0,-$H$40/(-$H$40+100),100/($H$40+100)))</f>
@@ -21604,7 +21604,7 @@
       </c>
       <c r="N40" s="19" t="inlineStr">
         <is>
-          <t>Model 42.3% (fair +136). Your call.</t>
+          <t>Model 42.0% (fair +138). Your call.</t>
         </is>
       </c>
       <c r="O40" s="15" t="n"/>
@@ -21613,405 +21613,9 @@
         <v/>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="12" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>New York Liberty @ Golden State Valkyries</t>
-        </is>
-      </c>
-      <c r="C41" s="12" t="inlineStr">
-        <is>
-          <t>23:00</t>
-        </is>
-      </c>
-      <c r="D41" s="12" t="inlineStr">
-        <is>
-          <t>Moneyline</t>
-        </is>
-      </c>
-      <c r="E41" s="12" t="inlineStr">
-        <is>
-          <t>New York Liberty</t>
-        </is>
-      </c>
-      <c r="F41" s="13" t="n">
-        <v>0.4216826923076923</v>
-      </c>
-      <c r="G41" s="14" t="n">
-        <v>137</v>
-      </c>
-      <c r="H41" s="15" t="n">
-        <v>108</v>
-      </c>
-      <c r="I41" s="13">
-        <f>IF($H$41="","",IF($H$41&lt;0,-$H$41/(-$H$41+100),100/($H$41+100)))</f>
-        <v/>
-      </c>
-      <c r="J41" s="16">
-        <f>IF($H$41="","",$F$41*IF($H$41&lt;0,-100/$H$41,$H$41/100)-(1-$F$41))</f>
-        <v/>
-      </c>
-      <c r="K41" s="17">
-        <f>IF($H$41="","",MAX(0,($F$41*IF($H$41&lt;0,-100/$H$41,$H$41/100)-(1-$F$41))/IF($H$41&lt;0,-100/$H$41,$H$41/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L41" s="18">
-        <f>IF($H$41="","",ROUND(MIN($K$41,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M41" s="12">
-        <f>IF($J$41="","",IF($J$41&lt;0,"Pass",IF($J$41&lt;'Settings'!$B$4,"Thin",IF($J$41&lt;0.06,"✅ Sharp band",IF($J$41&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N41" s="19" t="inlineStr">
-        <is>
-          <t>Model 42.2% (fair +137). Your call.</t>
-        </is>
-      </c>
-      <c r="O41" s="15" t="n"/>
-      <c r="P41" s="16">
-        <f>IF(OR($H$41="",$O$41=""),"",(1+IF($H$41&lt;0,-100/$H$41,$H$41/100))/(1+IF($O$41&lt;0,-100/$O$41,$O$41/100))-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="20" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="B42" s="20" t="inlineStr">
-        <is>
-          <t>New York Liberty @ Golden State Valkyries</t>
-        </is>
-      </c>
-      <c r="C42" s="20" t="inlineStr">
-        <is>
-          <t>23:00</t>
-        </is>
-      </c>
-      <c r="D42" s="20" t="inlineStr">
-        <is>
-          <t>Moneyline</t>
-        </is>
-      </c>
-      <c r="E42" s="20" t="inlineStr">
-        <is>
-          <t>Golden State Valkyries</t>
-        </is>
-      </c>
-      <c r="F42" s="13" t="n">
-        <v>0.578321568627451</v>
-      </c>
-      <c r="G42" s="14" t="n">
-        <v>-137</v>
-      </c>
-      <c r="H42" s="15" t="n">
-        <v>-104</v>
-      </c>
-      <c r="I42" s="13">
-        <f>IF($H$42="","",IF($H$42&lt;0,-$H$42/(-$H$42+100),100/($H$42+100)))</f>
-        <v/>
-      </c>
-      <c r="J42" s="16">
-        <f>IF($H$42="","",$F$42*IF($H$42&lt;0,-100/$H$42,$H$42/100)-(1-$F$42))</f>
-        <v/>
-      </c>
-      <c r="K42" s="17">
-        <f>IF($H$42="","",MAX(0,($F$42*IF($H$42&lt;0,-100/$H$42,$H$42/100)-(1-$F$42))/IF($H$42&lt;0,-100/$H$42,$H$42/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L42" s="18">
-        <f>IF($H$42="","",ROUND(MIN($K$42,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M42" s="12">
-        <f>IF($J$42="","",IF($J$42&lt;0,"Pass",IF($J$42&lt;'Settings'!$B$4,"Thin",IF($J$42&lt;0.06,"✅ Sharp band",IF($J$42&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N42" s="19" t="inlineStr">
-        <is>
-          <t>Model 57.8% (fair -137). Your call.</t>
-        </is>
-      </c>
-      <c r="O42" s="15" t="n"/>
-      <c r="P42" s="16">
-        <f>IF(OR($H$42="",$O$42=""),"",(1+IF($H$42&lt;0,-100/$H$42,$H$42/100))/(1+IF($O$42&lt;0,-100/$O$42,$O$42/100))-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="12" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>New York Liberty @ Golden State Valkyries</t>
-        </is>
-      </c>
-      <c r="C43" s="12" t="inlineStr">
-        <is>
-          <t>23:00</t>
-        </is>
-      </c>
-      <c r="D43" s="12" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="E43" s="12" t="inlineStr">
-        <is>
-          <t>Over 163.5</t>
-        </is>
-      </c>
-      <c r="F43" s="13" t="n">
-        <v>0.5769238095238095</v>
-      </c>
-      <c r="G43" s="14" t="n">
-        <v>-136</v>
-      </c>
-      <c r="H43" s="15" t="n">
-        <v>-110</v>
-      </c>
-      <c r="I43" s="13">
-        <f>IF($H$43="","",IF($H$43&lt;0,-$H$43/(-$H$43+100),100/($H$43+100)))</f>
-        <v/>
-      </c>
-      <c r="J43" s="16">
-        <f>IF($H$43="","",$F$43*IF($H$43&lt;0,-100/$H$43,$H$43/100)-(1-$F$43))</f>
-        <v/>
-      </c>
-      <c r="K43" s="17">
-        <f>IF($H$43="","",MAX(0,($F$43*IF($H$43&lt;0,-100/$H$43,$H$43/100)-(1-$F$43))/IF($H$43&lt;0,-100/$H$43,$H$43/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L43" s="18">
-        <f>IF($H$43="","",ROUND(MIN($K$43,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M43" s="12">
-        <f>IF($J$43="","",IF($J$43&lt;0,"Pass",IF($J$43&lt;'Settings'!$B$4,"Thin",IF($J$43&lt;0.06,"✅ Sharp band",IF($J$43&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N43" s="19" t="inlineStr">
-        <is>
-          <t>Model 57.7% (fair -136). Your call.</t>
-        </is>
-      </c>
-      <c r="O43" s="15" t="n"/>
-      <c r="P43" s="16">
-        <f>IF(OR($H$43="",$O$43=""),"",(1+IF($H$43&lt;0,-100/$H$43,$H$43/100))/(1+IF($O$43&lt;0,-100/$O$43,$O$43/100))-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="20" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="B44" s="20" t="inlineStr">
-        <is>
-          <t>New York Liberty @ Golden State Valkyries</t>
-        </is>
-      </c>
-      <c r="C44" s="20" t="inlineStr">
-        <is>
-          <t>23:00</t>
-        </is>
-      </c>
-      <c r="D44" s="20" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="E44" s="20" t="inlineStr">
-        <is>
-          <t>Under 163.5</t>
-        </is>
-      </c>
-      <c r="F44" s="13" t="n">
-        <v>0.4231</v>
-      </c>
-      <c r="G44" s="14" t="n">
-        <v>136</v>
-      </c>
-      <c r="H44" s="15" t="n">
-        <v>-110</v>
-      </c>
-      <c r="I44" s="13">
-        <f>IF($H$44="","",IF($H$44&lt;0,-$H$44/(-$H$44+100),100/($H$44+100)))</f>
-        <v/>
-      </c>
-      <c r="J44" s="16">
-        <f>IF($H$44="","",$F$44*IF($H$44&lt;0,-100/$H$44,$H$44/100)-(1-$F$44))</f>
-        <v/>
-      </c>
-      <c r="K44" s="17">
-        <f>IF($H$44="","",MAX(0,($F$44*IF($H$44&lt;0,-100/$H$44,$H$44/100)-(1-$F$44))/IF($H$44&lt;0,-100/$H$44,$H$44/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L44" s="18">
-        <f>IF($H$44="","",ROUND(MIN($K$44,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M44" s="12">
-        <f>IF($J$44="","",IF($J$44&lt;0,"Pass",IF($J$44&lt;'Settings'!$B$4,"Thin",IF($J$44&lt;0.06,"✅ Sharp band",IF($J$44&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N44" s="19" t="inlineStr">
-        <is>
-          <t>Model 42.3% (fair +136). Your call.</t>
-        </is>
-      </c>
-      <c r="O44" s="15" t="n"/>
-      <c r="P44" s="16">
-        <f>IF(OR($H$44="",$O$44=""),"",(1+IF($H$44&lt;0,-100/$H$44,$H$44/100))/(1+IF($O$44&lt;0,-100/$O$44,$O$44/100))-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="12" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>New York Liberty @ Golden State Valkyries</t>
-        </is>
-      </c>
-      <c r="C45" s="12" t="inlineStr">
-        <is>
-          <t>23:00</t>
-        </is>
-      </c>
-      <c r="D45" s="12" t="inlineStr">
-        <is>
-          <t>Spread</t>
-        </is>
-      </c>
-      <c r="E45" s="12" t="inlineStr">
-        <is>
-          <t>Golden State Valkyries +1.5</t>
-        </is>
-      </c>
-      <c r="F45" s="13" t="n">
-        <v>0.576435294117647</v>
-      </c>
-      <c r="G45" s="14" t="n">
-        <v>-136</v>
-      </c>
-      <c r="H45" s="15" t="n">
-        <v>-104</v>
-      </c>
-      <c r="I45" s="13">
-        <f>IF($H$45="","",IF($H$45&lt;0,-$H$45/(-$H$45+100),100/($H$45+100)))</f>
-        <v/>
-      </c>
-      <c r="J45" s="16">
-        <f>IF($H$45="","",$F$45*IF($H$45&lt;0,-100/$H$45,$H$45/100)-(1-$F$45))</f>
-        <v/>
-      </c>
-      <c r="K45" s="17">
-        <f>IF($H$45="","",MAX(0,($F$45*IF($H$45&lt;0,-100/$H$45,$H$45/100)-(1-$F$45))/IF($H$45&lt;0,-100/$H$45,$H$45/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L45" s="18">
-        <f>IF($H$45="","",ROUND(MIN($K$45,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M45" s="12">
-        <f>IF($J$45="","",IF($J$45&lt;0,"Pass",IF($J$45&lt;'Settings'!$B$4,"Thin",IF($J$45&lt;0.06,"✅ Sharp band",IF($J$45&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N45" s="19" t="inlineStr">
-        <is>
-          <t>Model 57.6% (fair -136). Your call.</t>
-        </is>
-      </c>
-      <c r="O45" s="15" t="n"/>
-      <c r="P45" s="16">
-        <f>IF(OR($H$45="",$O$45=""),"",(1+IF($H$45&lt;0,-100/$H$45,$H$45/100))/(1+IF($O$45&lt;0,-100/$O$45,$O$45/100))-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="20" t="inlineStr">
-        <is>
-          <t>2026-06-28</t>
-        </is>
-      </c>
-      <c r="B46" s="20" t="inlineStr">
-        <is>
-          <t>New York Liberty @ Golden State Valkyries</t>
-        </is>
-      </c>
-      <c r="C46" s="20" t="inlineStr">
-        <is>
-          <t>23:00</t>
-        </is>
-      </c>
-      <c r="D46" s="20" t="inlineStr">
-        <is>
-          <t>Spread</t>
-        </is>
-      </c>
-      <c r="E46" s="20" t="inlineStr">
-        <is>
-          <t>New York Liberty -1.5</t>
-        </is>
-      </c>
-      <c r="F46" s="13" t="n">
-        <v>0.42355</v>
-      </c>
-      <c r="G46" s="14" t="n">
-        <v>136</v>
-      </c>
-      <c r="H46" s="15" t="n">
-        <v>100</v>
-      </c>
-      <c r="I46" s="13">
-        <f>IF($H$46="","",IF($H$46&lt;0,-$H$46/(-$H$46+100),100/($H$46+100)))</f>
-        <v/>
-      </c>
-      <c r="J46" s="16">
-        <f>IF($H$46="","",$F$46*IF($H$46&lt;0,-100/$H$46,$H$46/100)-(1-$F$46))</f>
-        <v/>
-      </c>
-      <c r="K46" s="17">
-        <f>IF($H$46="","",MAX(0,($F$46*IF($H$46&lt;0,-100/$H$46,$H$46/100)-(1-$F$46))/IF($H$46&lt;0,-100/$H$46,$H$46/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L46" s="18">
-        <f>IF($H$46="","",ROUND(MIN($K$46,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M46" s="12">
-        <f>IF($J$46="","",IF($J$46&lt;0,"Pass",IF($J$46&lt;'Settings'!$B$4,"Thin",IF($J$46&lt;0.06,"✅ Sharp band",IF($J$46&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N46" s="19" t="inlineStr">
-        <is>
-          <t>Model 42.4% (fair +136). Your call.</t>
-        </is>
-      </c>
-      <c r="O46" s="15" t="n"/>
-      <c r="P46" s="16">
-        <f>IF(OR($H$46="",$O$46=""),"",(1+IF($H$46&lt;0,-100/$H$46,$H$46/100))/(1+IF($O$46&lt;0,-100/$O$46,$O$46/100))-1)</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J46">
+  <conditionalFormatting sqref="J5:J40">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -22115,28 +21719,28 @@
         </is>
       </c>
       <c r="B5" s="21" t="n">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C5" s="22" t="n">
-        <v>0.2503</v>
+        <v>0.2508</v>
       </c>
       <c r="D5" s="21" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E5" s="13" t="n">
-        <v>0.4639</v>
+        <v>0.4611</v>
       </c>
       <c r="F5" s="23" t="n">
-        <v>0.53</v>
+        <v>-0.47</v>
       </c>
       <c r="G5" s="24" t="n">
-        <v>0.32</v>
+        <v>-0.28</v>
       </c>
       <c r="H5" s="24" t="n">
-        <v>2.72</v>
+        <v>2.28</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>0.5068</v>
+        <v>0.5034</v>
       </c>
     </row>
     <row r="6">
@@ -22146,28 +21750,28 @@
         </is>
       </c>
       <c r="B6" s="21" t="n">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C6" s="22" t="n">
-        <v>0.2507</v>
+        <v>0.2512</v>
       </c>
       <c r="D6" s="21" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>0.5</v>
+        <v>0.4962</v>
       </c>
       <c r="F6" s="23" t="n">
-        <v>5.78</v>
+        <v>4.78</v>
       </c>
       <c r="G6" s="24" t="n">
-        <v>4.45</v>
+        <v>3.65</v>
       </c>
       <c r="H6" s="24" t="n">
-        <v>4.17</v>
+        <v>3.61</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>0.5339</v>
+        <v>0.5294</v>
       </c>
     </row>
     <row r="7">
@@ -22250,7 +21854,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>When the model said X%, how often it actually happened (n=191, ECE 0.069 — lower is better; a calibrated model's bars sit on the diagonal).</t>
+          <t>When the model said X%, how often it actually happened (n=193, ECE 0.063 — lower is better; a calibrated model's bars sit on the diagonal).</t>
         </is>
       </c>
     </row>
@@ -22345,16 +21949,16 @@
         </is>
       </c>
       <c r="B20" s="21" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>0.4543</v>
       </c>
       <c r="D20" s="13" t="n">
-        <v>0.4444</v>
+        <v>0.4531</v>
       </c>
       <c r="E20" s="26" t="n">
-        <v>-0.009900000000000001</v>
+        <v>-0.0012</v>
       </c>
     </row>
     <row r="21">
@@ -22364,16 +21968,16 @@
         </is>
       </c>
       <c r="B21" s="21" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C21" s="13" t="n">
-        <v>0.5431</v>
+        <v>0.5434</v>
       </c>
       <c r="D21" s="13" t="n">
-        <v>0.5735</v>
+        <v>0.5652</v>
       </c>
       <c r="E21" s="26" t="n">
-        <v>0.0304</v>
+        <v>0.0218</v>
       </c>
     </row>
     <row r="22">

</xml_diff>

<commit_message>
data: hourly update 2026-06-27 22:07Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-06-27.xlsx
+++ b/data/output/workbook/2026-06-27.xlsx
@@ -551,7 +551,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="9896475"/>
+    <ext cx="10125075" cy="9477375"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -954,7 +954,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-27 17:03</t>
+          <t>2026-06-27 18:07</t>
         </is>
       </c>
     </row>
@@ -4530,7 +4530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q77"/>
+  <dimension ref="A1:Q75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4547,823 +4547,823 @@
         </is>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" s="29" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks offense vs Tampa Bay Rays defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="30" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B62" s="30" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C62" s="30" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D62" s="30" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E62" s="30" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F62" s="30" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G62" s="30" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H62" s="30" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I62" s="30" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J62" s="30" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K62" s="30" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L62" s="30" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M62" s="30" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N62" s="30" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O62" s="30" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P62" s="30" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q62" s="30" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
+        </is>
+      </c>
+    </row>
     <row r="63">
-      <c r="A63" s="29" t="inlineStr">
-        <is>
-          <t>Arizona Diamondbacks offense vs Tampa Bay Rays defense</t>
+      <c r="A63" s="31" t="inlineStr">
+        <is>
+          <t>Runs/G</t>
+        </is>
+      </c>
+      <c r="B63" s="32" t="n">
+        <v>4.976</v>
+      </c>
+      <c r="C63" s="32" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="D63" s="32" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="E63" s="32" t="n">
+        <v>4.467</v>
+      </c>
+      <c r="F63" s="32" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="G63" s="32" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="H63" s="36" t="inlineStr">
+        <is>
+          <t>25th</t>
+        </is>
+      </c>
+      <c r="I63" s="32" t="inlineStr"/>
+      <c r="J63" s="36" t="inlineStr">
+        <is>
+          <t>26th</t>
+        </is>
+      </c>
+      <c r="K63" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="L63" s="32" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="M63" s="32" t="n">
+        <v>4.867</v>
+      </c>
+      <c r="N63" s="32" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="O63" s="32" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="P63" s="32" t="n">
+        <v>4.234</v>
+      </c>
+      <c r="Q63" s="35" t="inlineStr">
+        <is>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="30" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B64" s="30" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C64" s="30" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D64" s="30" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E64" s="30" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F64" s="30" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G64" s="30" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H64" s="30" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I64" s="30" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J64" s="30" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K64" s="30" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L64" s="30" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M64" s="30" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N64" s="30" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O64" s="30" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P64" s="30" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q64" s="30" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="A64" s="31" t="inlineStr">
+        <is>
+          <t>Hits/G</t>
+        </is>
+      </c>
+      <c r="B64" s="32" t="n">
+        <v>8.688000000000001</v>
+      </c>
+      <c r="C64" s="32" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="D64" s="32" t="n">
+        <v>8.85</v>
+      </c>
+      <c r="E64" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="F64" s="32" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="G64" s="32" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="H64" s="34" t="inlineStr">
+        <is>
+          <t>12th</t>
+        </is>
+      </c>
+      <c r="I64" s="32" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="J64" s="34" t="inlineStr">
+        <is>
+          <t>17th</t>
+        </is>
+      </c>
+      <c r="K64" s="32" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="L64" s="32" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="M64" s="32" t="n">
+        <v>8.067</v>
+      </c>
+      <c r="N64" s="32" t="n">
+        <v>8.050000000000001</v>
+      </c>
+      <c r="O64" s="32" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="P64" s="32" t="n">
+        <v>7.868</v>
+      </c>
+      <c r="Q64" s="35" t="inlineStr">
+        <is>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="31" t="inlineStr">
         <is>
-          <t>Runs/G</t>
+          <t>HR/G</t>
         </is>
       </c>
       <c r="B65" s="32" t="n">
-        <v>4.976</v>
+        <v>1.329</v>
       </c>
       <c r="C65" s="32" t="n">
-        <v>4.7</v>
+        <v>1.033</v>
       </c>
       <c r="D65" s="32" t="n">
-        <v>4.45</v>
+        <v>0.85</v>
       </c>
       <c r="E65" s="32" t="n">
-        <v>4.467</v>
+        <v>1</v>
       </c>
       <c r="F65" s="32" t="n">
-        <v>3.4</v>
+        <v>0.9</v>
       </c>
       <c r="G65" s="32" t="n">
-        <v>2.6</v>
+        <v>0.8</v>
       </c>
       <c r="H65" s="36" t="inlineStr">
         <is>
-          <t>25th</t>
+          <t>22nd</t>
         </is>
       </c>
       <c r="I65" s="32" t="inlineStr"/>
-      <c r="J65" s="36" t="inlineStr">
-        <is>
-          <t>26th</t>
-        </is>
-      </c>
-      <c r="K65" s="32" t="n">
-        <v>6</v>
-      </c>
-      <c r="L65" s="32" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="M65" s="32" t="n">
-        <v>4.867</v>
-      </c>
-      <c r="N65" s="32" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="O65" s="32" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="P65" s="32" t="n">
-        <v>4.234</v>
+      <c r="J65" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P65" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q65" s="35" t="inlineStr">
         <is>
-          <t>Opp Runs/G</t>
+          <t>Opp HR/G</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="31" t="inlineStr">
         <is>
-          <t>Hits/G</t>
+          <t>Batter K/G</t>
         </is>
       </c>
       <c r="B66" s="32" t="n">
-        <v>8.688000000000001</v>
+        <v>8.265000000000001</v>
       </c>
       <c r="C66" s="32" t="n">
+        <v>8.467000000000001</v>
+      </c>
+      <c r="D66" s="32" t="n">
+        <v>8.35</v>
+      </c>
+      <c r="E66" s="32" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="F66" s="32" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="G66" s="32" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="H66" s="36" t="inlineStr">
+        <is>
+          <t>23rd</t>
+        </is>
+      </c>
+      <c r="I66" s="32" t="inlineStr"/>
+      <c r="J66" s="34" t="inlineStr">
+        <is>
+          <t>15th</t>
+        </is>
+      </c>
+      <c r="K66" s="32" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="L66" s="32" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="D66" s="32" t="n">
-        <v>8.85</v>
-      </c>
-      <c r="E66" s="32" t="n">
-        <v>9</v>
-      </c>
-      <c r="F66" s="32" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="G66" s="32" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="H66" s="34" t="inlineStr">
-        <is>
-          <t>12th</t>
-        </is>
-      </c>
-      <c r="I66" s="32" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="J66" s="34" t="inlineStr">
-        <is>
-          <t>17th</t>
-        </is>
-      </c>
-      <c r="K66" s="32" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="L66" s="32" t="n">
-        <v>8.4</v>
-      </c>
       <c r="M66" s="32" t="n">
-        <v>8.067</v>
+        <v>8.333</v>
       </c>
       <c r="N66" s="32" t="n">
-        <v>8.050000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="O66" s="32" t="n">
-        <v>7.8</v>
+        <v>9.5</v>
       </c>
       <c r="P66" s="32" t="n">
-        <v>7.868</v>
+        <v>8.737</v>
       </c>
       <c r="Q66" s="35" t="inlineStr">
         <is>
-          <t>Opp Hits/G</t>
+          <t>Opp Batter K/G</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>1st Inn R/G</t>
         </is>
       </c>
       <c r="B67" s="32" t="n">
-        <v>1.329</v>
+        <v>0.612</v>
       </c>
       <c r="C67" s="32" t="n">
-        <v>1.033</v>
+        <v>0.467</v>
       </c>
       <c r="D67" s="32" t="n">
-        <v>0.85</v>
+        <v>0.5</v>
       </c>
       <c r="E67" s="32" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="F67" s="32" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="G67" s="32" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H67" s="33" t="inlineStr">
+        <is>
+          <t>10th</t>
+        </is>
+      </c>
+      <c r="I67" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J67" s="36" t="inlineStr">
+        <is>
+          <t>25th</t>
+        </is>
+      </c>
+      <c r="K67" s="32" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="L67" s="32" t="n">
         <v>0.8</v>
       </c>
-      <c r="H67" s="36" t="inlineStr">
-        <is>
-          <t>22nd</t>
-        </is>
-      </c>
-      <c r="I67" s="32" t="inlineStr"/>
-      <c r="J67" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K67" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L67" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M67" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N67" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O67" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P67" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="M67" s="32" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="N67" s="32" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="O67" s="32" t="n">
+        <v>0.467</v>
+      </c>
+      <c r="P67" s="32" t="n">
+        <v>0.473</v>
       </c>
       <c r="Q67" s="35" t="inlineStr">
         <is>
-          <t>Opp HR/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="31" t="inlineStr">
-        <is>
-          <t>Batter K/G</t>
-        </is>
-      </c>
-      <c r="B68" s="32" t="n">
-        <v>8.265000000000001</v>
-      </c>
-      <c r="C68" s="32" t="n">
-        <v>8.467000000000001</v>
-      </c>
-      <c r="D68" s="32" t="n">
-        <v>8.35</v>
-      </c>
-      <c r="E68" s="32" t="n">
+          <t>Opp 1st Inn R/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="29" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays offense vs Arizona Diamondbacks defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="30" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B70" s="30" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C70" s="30" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D70" s="30" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E70" s="30" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F70" s="30" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G70" s="30" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H70" s="30" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I70" s="30" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J70" s="30" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K70" s="30" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L70" s="30" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M70" s="30" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N70" s="30" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O70" s="30" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P70" s="30" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q70" s="30" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="31" t="inlineStr">
+        <is>
+          <t>Runs/G</t>
+        </is>
+      </c>
+      <c r="B71" s="32" t="n">
+        <v>4.437</v>
+      </c>
+      <c r="C71" s="32" t="n">
+        <v>4.033</v>
+      </c>
+      <c r="D71" s="32" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="E71" s="32" t="n">
+        <v>3.667</v>
+      </c>
+      <c r="F71" s="32" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="G71" s="32" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="H71" s="34" t="inlineStr">
+        <is>
+          <t>14th</t>
+        </is>
+      </c>
+      <c r="I71" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J71" s="36" t="inlineStr">
+        <is>
+          <t>30th</t>
+        </is>
+      </c>
+      <c r="K71" s="32" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="L71" s="32" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="M71" s="32" t="n">
+        <v>5.333</v>
+      </c>
+      <c r="N71" s="32" t="n">
+        <v>5.35</v>
+      </c>
+      <c r="O71" s="32" t="n">
+        <v>4.767</v>
+      </c>
+      <c r="P71" s="32" t="n">
+        <v>4.847</v>
+      </c>
+      <c r="Q71" s="35" t="inlineStr">
+        <is>
+          <t>Opp Runs/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="31" t="inlineStr">
+        <is>
+          <t>Hits/G</t>
+        </is>
+      </c>
+      <c r="B72" s="32" t="n">
+        <v>8.521000000000001</v>
+      </c>
+      <c r="C72" s="32" t="n">
         <v>8.4</v>
       </c>
-      <c r="F68" s="32" t="n">
-        <v>8.6</v>
-      </c>
-      <c r="G68" s="32" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="H68" s="36" t="inlineStr">
-        <is>
-          <t>23rd</t>
-        </is>
-      </c>
-      <c r="I68" s="32" t="inlineStr"/>
-      <c r="J68" s="34" t="inlineStr">
-        <is>
-          <t>15th</t>
-        </is>
-      </c>
-      <c r="K68" s="32" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="L68" s="32" t="n">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="M68" s="32" t="n">
-        <v>8.333</v>
-      </c>
-      <c r="N68" s="32" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="O68" s="32" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="P68" s="32" t="n">
-        <v>8.737</v>
-      </c>
-      <c r="Q68" s="35" t="inlineStr">
-        <is>
-          <t>Opp Batter K/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="31" t="inlineStr">
-        <is>
-          <t>1st Inn R/G</t>
-        </is>
-      </c>
-      <c r="B69" s="32" t="n">
-        <v>0.612</v>
-      </c>
-      <c r="C69" s="32" t="n">
-        <v>0.467</v>
-      </c>
-      <c r="D69" s="32" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E69" s="32" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="F69" s="32" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="G69" s="32" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H69" s="33" t="inlineStr">
-        <is>
-          <t>10th</t>
-        </is>
-      </c>
-      <c r="I69" s="32" t="inlineStr">
+      <c r="D72" s="32" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="E72" s="32" t="n">
+        <v>8.667</v>
+      </c>
+      <c r="F72" s="32" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="G72" s="32" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H72" s="33" t="inlineStr">
+        <is>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="I72" s="32" t="inlineStr">
         <is>
           <t>★★★</t>
         </is>
       </c>
-      <c r="J69" s="36" t="inlineStr">
-        <is>
-          <t>25th</t>
-        </is>
-      </c>
-      <c r="K69" s="32" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="L69" s="32" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="M69" s="32" t="n">
-        <v>0.667</v>
-      </c>
-      <c r="N69" s="32" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="O69" s="32" t="n">
-        <v>0.467</v>
-      </c>
-      <c r="P69" s="32" t="n">
-        <v>0.473</v>
-      </c>
-      <c r="Q69" s="35" t="inlineStr">
-        <is>
-          <t>Opp 1st Inn R/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="29" t="inlineStr">
-        <is>
-          <t>Tampa Bay Rays offense vs Arizona Diamondbacks defense</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="30" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B72" s="30" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C72" s="30" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D72" s="30" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E72" s="30" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F72" s="30" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G72" s="30" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H72" s="30" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I72" s="30" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J72" s="30" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K72" s="30" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L72" s="30" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M72" s="30" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N72" s="30" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O72" s="30" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P72" s="30" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q72" s="30" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="J72" s="36" t="inlineStr">
+        <is>
+          <t>27th</t>
+        </is>
+      </c>
+      <c r="K72" s="32" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="L72" s="32" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="M72" s="32" t="n">
+        <v>9.132999999999999</v>
+      </c>
+      <c r="N72" s="32" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="O72" s="32" t="n">
+        <v>8.567</v>
+      </c>
+      <c r="P72" s="32" t="n">
+        <v>8.840999999999999</v>
+      </c>
+      <c r="Q72" s="35" t="inlineStr">
+        <is>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="31" t="inlineStr">
         <is>
-          <t>Runs/G</t>
+          <t>HR/G</t>
         </is>
       </c>
       <c r="B73" s="32" t="n">
-        <v>4.437</v>
+        <v>1.114</v>
       </c>
       <c r="C73" s="32" t="n">
-        <v>4.033</v>
+        <v>1.133</v>
       </c>
       <c r="D73" s="32" t="n">
-        <v>3.55</v>
+        <v>1.15</v>
       </c>
       <c r="E73" s="32" t="n">
-        <v>3.667</v>
+        <v>1</v>
       </c>
       <c r="F73" s="32" t="n">
-        <v>3.9</v>
+        <v>1</v>
       </c>
       <c r="G73" s="32" t="n">
-        <v>3.6</v>
+        <v>1</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
-          <t>14th</t>
-        </is>
-      </c>
-      <c r="I73" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J73" s="36" t="inlineStr">
-        <is>
-          <t>30th</t>
-        </is>
-      </c>
-      <c r="K73" s="32" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="L73" s="32" t="n">
-        <v>5.9</v>
-      </c>
-      <c r="M73" s="32" t="n">
-        <v>5.333</v>
-      </c>
-      <c r="N73" s="32" t="n">
-        <v>5.35</v>
-      </c>
-      <c r="O73" s="32" t="n">
-        <v>4.767</v>
-      </c>
-      <c r="P73" s="32" t="n">
-        <v>4.847</v>
+          <t>17th</t>
+        </is>
+      </c>
+      <c r="I73" s="32" t="inlineStr"/>
+      <c r="J73" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P73" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q73" s="35" t="inlineStr">
         <is>
-          <t>Opp Runs/G</t>
+          <t>Opp HR/G</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="31" t="inlineStr">
         <is>
-          <t>Hits/G</t>
+          <t>Batter K/G</t>
         </is>
       </c>
       <c r="B74" s="32" t="n">
-        <v>8.521000000000001</v>
+        <v>8.611000000000001</v>
       </c>
       <c r="C74" s="32" t="n">
-        <v>8.4</v>
+        <v>8.967000000000001</v>
       </c>
       <c r="D74" s="32" t="n">
-        <v>8.300000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="E74" s="32" t="n">
-        <v>8.667</v>
+        <v>9.667</v>
       </c>
       <c r="F74" s="32" t="n">
-        <v>8.5</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G74" s="32" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="H74" s="33" t="inlineStr">
-        <is>
-          <t>3rd</t>
-        </is>
-      </c>
-      <c r="I74" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J74" s="36" t="inlineStr">
-        <is>
-          <t>27th</t>
+        <v>10.2</v>
+      </c>
+      <c r="H74" s="34" t="inlineStr">
+        <is>
+          <t>18th</t>
+        </is>
+      </c>
+      <c r="I74" s="32" t="inlineStr"/>
+      <c r="J74" s="34" t="inlineStr">
+        <is>
+          <t>16th</t>
         </is>
       </c>
       <c r="K74" s="32" t="n">
-        <v>10.4</v>
+        <v>9.4</v>
       </c>
       <c r="L74" s="32" t="n">
-        <v>9.800000000000001</v>
+        <v>9</v>
       </c>
       <c r="M74" s="32" t="n">
-        <v>9.132999999999999</v>
+        <v>8.333</v>
       </c>
       <c r="N74" s="32" t="n">
-        <v>8.75</v>
+        <v>7.9</v>
       </c>
       <c r="O74" s="32" t="n">
-        <v>8.567</v>
+        <v>7.8</v>
       </c>
       <c r="P74" s="32" t="n">
-        <v>8.840999999999999</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="Q74" s="35" t="inlineStr">
         <is>
-          <t>Opp Hits/G</t>
+          <t>Opp Batter K/G</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="31" t="inlineStr">
         <is>
-          <t>HR/G</t>
+          <t>1st Inn R/G</t>
         </is>
       </c>
       <c r="B75" s="32" t="n">
-        <v>1.114</v>
+        <v>0.587</v>
       </c>
       <c r="C75" s="32" t="n">
-        <v>1.133</v>
+        <v>0.867</v>
       </c>
       <c r="D75" s="32" t="n">
-        <v>1.15</v>
+        <v>0.7</v>
       </c>
       <c r="E75" s="32" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="F75" s="32" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G75" s="32" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H75" s="34" t="inlineStr">
+        <is>
+          <t>16th</t>
+        </is>
+      </c>
+      <c r="I75" s="32" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J75" s="36" t="inlineStr">
+        <is>
+          <t>29th</t>
+        </is>
+      </c>
+      <c r="K75" s="32" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="L75" s="32" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="M75" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="F75" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G75" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="H75" s="34" t="inlineStr">
-        <is>
-          <t>17th</t>
-        </is>
-      </c>
-      <c r="I75" s="32" t="inlineStr"/>
-      <c r="J75" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K75" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L75" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M75" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N75" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O75" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P75" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="N75" s="32" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="O75" s="32" t="n">
+        <v>0.733</v>
+      </c>
+      <c r="P75" s="32" t="n">
+        <v>0.641</v>
       </c>
       <c r="Q75" s="35" t="inlineStr">
-        <is>
-          <t>Opp HR/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="31" t="inlineStr">
-        <is>
-          <t>Batter K/G</t>
-        </is>
-      </c>
-      <c r="B76" s="32" t="n">
-        <v>8.611000000000001</v>
-      </c>
-      <c r="C76" s="32" t="n">
-        <v>8.967000000000001</v>
-      </c>
-      <c r="D76" s="32" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="E76" s="32" t="n">
-        <v>9.667</v>
-      </c>
-      <c r="F76" s="32" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="G76" s="32" t="n">
-        <v>10.2</v>
-      </c>
-      <c r="H76" s="34" t="inlineStr">
-        <is>
-          <t>18th</t>
-        </is>
-      </c>
-      <c r="I76" s="32" t="inlineStr"/>
-      <c r="J76" s="34" t="inlineStr">
-        <is>
-          <t>16th</t>
-        </is>
-      </c>
-      <c r="K76" s="32" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="L76" s="32" t="n">
-        <v>9</v>
-      </c>
-      <c r="M76" s="32" t="n">
-        <v>8.333</v>
-      </c>
-      <c r="N76" s="32" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="O76" s="32" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="P76" s="32" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="Q76" s="35" t="inlineStr">
-        <is>
-          <t>Opp Batter K/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="31" t="inlineStr">
-        <is>
-          <t>1st Inn R/G</t>
-        </is>
-      </c>
-      <c r="B77" s="32" t="n">
-        <v>0.587</v>
-      </c>
-      <c r="C77" s="32" t="n">
-        <v>0.867</v>
-      </c>
-      <c r="D77" s="32" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="E77" s="32" t="n">
-        <v>0.667</v>
-      </c>
-      <c r="F77" s="32" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G77" s="32" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="H77" s="34" t="inlineStr">
-        <is>
-          <t>16th</t>
-        </is>
-      </c>
-      <c r="I77" s="32" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J77" s="36" t="inlineStr">
-        <is>
-          <t>29th</t>
-        </is>
-      </c>
-      <c r="K77" s="32" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="L77" s="32" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="M77" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="N77" s="32" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="O77" s="32" t="n">
-        <v>0.733</v>
-      </c>
-      <c r="P77" s="32" t="n">
-        <v>0.641</v>
-      </c>
-      <c r="Q77" s="35" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
@@ -8108,37 +8108,37 @@
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Indiana Fever</t>
+          <t>Cincinnati Reds @ Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Over 179.5</t>
+          <t>Pittsburgh Pirates -1.5</t>
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.715</v>
+        <v>0.5008208955223882</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-251</v>
+        <v>-100</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>-104</v>
+        <v>168</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -8162,7 +8162,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 71.5% (fair -251). Your call.</t>
+          <t>Model 50.1% (fair -100). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -8174,37 +8174,37 @@
     <row r="6">
       <c r="A6" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Pittsburgh Pirates</t>
+          <t>Los Angeles Sparks @ Indiana Fever</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates -1.5</t>
+          <t>Over 181.5</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.4966544117647059</v>
+        <v>0.6680980392156862</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>101</v>
+        <v>-201</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>172</v>
+        <v>-104</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -8228,7 +8228,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 49.7% (fair +101). Your call.</t>
+          <t>Model 66.8% (fair -201). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -8311,12 +8311,12 @@
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Washington Nationals @ Baltimore Orioles</t>
+          <t>Portland Fire @ Washington Mystics</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
@@ -8326,17 +8326,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Over 9.5</t>
+          <t>Over 166.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5857560975609757</v>
+        <v>0.5774509803921568</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-141</v>
+        <v>-137</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -8360,7 +8360,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 58.6% (fair -141). Your call.</t>
+          <t>Model 57.7% (fair -137). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -8377,12 +8377,12 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Portland Fire @ Washington Mystics</t>
+          <t>Houston Astros @ Detroit Tigers</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -8392,17 +8392,17 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Over 166.5</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.5774509803921568</v>
+        <v>0.5749</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-137</v>
+        <v>-135</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -8426,7 +8426,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -137). Your call.</t>
+          <t>Model 57.5% (fair -135). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -8438,37 +8438,37 @@
     <row r="10">
       <c r="A10" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Houston Astros @ Detroit Tigers</t>
+          <t>Cincinnati Reds @ Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5746</v>
+        <v>0.5560194174757281</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-135</v>
+        <v>-125</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -8492,7 +8492,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 57.5% (fair -135). Your call.</t>
+          <t>Model 55.6% (fair -125). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -8509,32 +8509,32 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Kansas City Royals @ Chicago White Sox</t>
+          <t>New York Liberty @ Golden State Valkyries</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Over 9</t>
+          <t>Golden State Valkyries</t>
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.5866682926829269</v>
+        <v>0.578321568627451</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-142</v>
+        <v>-137</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>-105</v>
+        <v>-104</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -8558,7 +8558,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 58.7% (fair -142). Your call.</t>
+          <t>Model 57.8% (fair -137). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -8570,37 +8570,37 @@
     <row r="12">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Pittsburgh Pirates</t>
+          <t>Washington Nationals @ Baltimore Orioles</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="D12" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Baltimore Orioles -1.5</t>
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.5560194174757281</v>
+        <v>0.5262264150943395</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-125</v>
+        <v>-111</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -8624,7 +8624,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 55.6% (fair -125). Your call.</t>
+          <t>Model 52.6% (fair -111). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -8641,32 +8641,32 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>New York Liberty @ Golden State Valkyries</t>
+          <t>Arizona Diamondbacks @ Tampa Bay Rays</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Golden State Valkyries +1.5</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5795450980392156</v>
+        <v>0.5958069767441861</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-138</v>
+        <v>-147</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>-104</v>
+        <v>-115</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -8690,7 +8690,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 58.0% (fair -138). Your call.</t>
+          <t>Model 59.6% (fair -147). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -8707,12 +8707,12 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>New York Liberty @ Golden State Valkyries</t>
+          <t>Washington Nationals @ Baltimore Orioles</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
@@ -8722,17 +8722,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Golden State Valkyries</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.578321568627451</v>
+        <v>0.6854057034220533</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-137</v>
+        <v>-218</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>-104</v>
+        <v>-163</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -8756,7 +8756,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 57.8% (fair -137). Your call.</t>
+          <t>Model 68.5% (fair -218). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -8773,32 +8773,32 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Seattle Mariners @ Cleveland Guardians</t>
+          <t>Las Vegas Aces @ Chicago Sky</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Over 178.5</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.54375</v>
+        <v>0.55275</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-119</v>
+        <v>-124</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -8822,7 +8822,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 54.4% (fair -119). Your call.</t>
+          <t>Model 55.3% (fair -124). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -8839,12 +8839,12 @@
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks @ Tampa Bay Rays</t>
+          <t>Texas Rangers @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
@@ -8854,17 +8854,17 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.5958069767441861</v>
+        <v>0.55175</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-147</v>
+        <v>-123</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>-115</v>
+        <v>100</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -8888,7 +8888,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 59.6% (fair -147). Your call.</t>
+          <t>Model 55.2% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -8924,13 +8924,13 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.5767615384615384</v>
+        <v>0.5778666666666666</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-136</v>
+        <v>-137</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>-108</v>
+        <v>-110</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -8954,7 +8954,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -136). Your call.</t>
+          <t>Model 57.8% (fair -137). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -8971,32 +8971,32 @@
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>Washington Nationals @ Baltimore Orioles</t>
+          <t>New York Liberty @ Golden State Valkyries</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>Baltimore Orioles -1.5</t>
+          <t>Over 163.5</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5273809523809523</v>
+        <v>0.5769238095238095</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-112</v>
+        <v>-136</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>110</v>
+        <v>-110</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -9020,7 +9020,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 52.7% (fair -112). Your call.</t>
+          <t>Model 57.7% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -9037,32 +9037,32 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Washington Nationals @ Baltimore Orioles</t>
+          <t>Atlanta Braves @ San Francisco Giants</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.6854057034220533</v>
+        <v>0.5606823529411765</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-218</v>
+        <v>-128</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>-163</v>
+        <v>-104</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -9086,7 +9086,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 68.5% (fair -218). Your call.</t>
+          <t>Model 56.1% (fair -128). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -9103,29 +9103,29 @@
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>Las Vegas Aces @ Chicago Sky</t>
+          <t>Seattle Mariners @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Over 178.5</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.55275</v>
+        <v>0.54865</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>-124</v>
+        <v>-122</v>
       </c>
       <c r="H20" s="15" t="n">
         <v>100</v>
@@ -9152,7 +9152,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 55.3% (fair -124). Your call.</t>
+          <t>Model 54.9% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -9164,37 +9164,37 @@
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Toronto Blue Jays</t>
+          <t>Washington Nationals @ Baltimore Orioles</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.55175</v>
+        <v>0.5517098039215687</v>
       </c>
       <c r="G21" s="14" t="n">
         <v>-123</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>100</v>
+        <v>-104</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -9230,37 +9230,37 @@
     <row r="22">
       <c r="A22" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>New York Liberty @ Golden State Valkyries</t>
+          <t>Chicago Cubs @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C22" s="20" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D22" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Over 163.5</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.5769238095238095</v>
+        <v>0.6313406639004149</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-136</v>
+        <v>-171</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>-110</v>
+        <v>-141</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -9284,7 +9284,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -136). Your call.</t>
+          <t>Model 63.1% (fair -171). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -9296,37 +9296,37 @@
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>Atlanta Braves @ San Francisco Giants</t>
+          <t>Seattle Mariners @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.5636707317073171</v>
+        <v>0.6175531914893617</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>-129</v>
+        <v>-161</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>-105</v>
+        <v>-135</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -9350,7 +9350,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 56.4% (fair -129). Your call.</t>
+          <t>Model 61.8% (fair -161). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -9367,12 +9367,12 @@
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>Washington Nationals @ Baltimore Orioles</t>
+          <t>Arizona Diamondbacks @ Tampa Bay Rays</t>
         </is>
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
-          <t>23:05</t>
+          <t>22:10</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
@@ -9382,17 +9382,17 @@
       </c>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Arizona Diamondbacks</t>
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5510470588235293</v>
+        <v>0.4763555555555556</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-123</v>
+        <v>110</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>-104</v>
+        <v>125</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -9416,7 +9416,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 55.1% (fair -123). Your call.</t>
+          <t>Model 47.6% (fair +110). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -9428,37 +9428,37 @@
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks @ Tampa Bay Rays</t>
+          <t>Colorado Rockies @ Minnesota Twins</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>22:10</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Over 9</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.4752863436123348</v>
+        <v>0.53585</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>110</v>
+        <v>-115</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -9482,7 +9482,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 47.5% (fair +110). Your call.</t>
+          <t>Model 53.6% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -9499,12 +9499,12 @@
       </c>
       <c r="B26" s="20" t="inlineStr">
         <is>
-          <t>Kansas City Royals @ Chicago White Sox</t>
+          <t>Atlanta Braves @ San Francisco Giants</t>
         </is>
       </c>
       <c r="C26" s="20" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="D26" s="20" t="inlineStr">
@@ -9514,17 +9514,17 @@
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Chicago White Sox -1.5</t>
+          <t>San Francisco Giants +1.5</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4223529411764706</v>
+        <v>0.6048391304347827</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>137</v>
+        <v>-153</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>155</v>
+        <v>-130</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -9548,7 +9548,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 42.2% (fair +137). Your call.</t>
+          <t>Model 60.5% (fair -153). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -9565,32 +9565,32 @@
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>New York Yankees @ Boston Red Sox</t>
+          <t>New York Liberty @ Golden State Valkyries</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>23:20</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Under 9</t>
+          <t>Golden State Valkyries -1.5</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.5172596153846154</v>
+        <v>0.5218536585365855</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>-107</v>
+        <v>-109</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -9614,7 +9614,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 51.7% (fair -107). Your call.</t>
+          <t>Model 52.2% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -9626,37 +9626,37 @@
     <row r="28">
       <c r="A28" s="20" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>Colorado Rockies @ Minnesota Twins</t>
+          <t>Philadelphia Phillies @ New York Mets</t>
         </is>
       </c>
       <c r="C28" s="20" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>20:10</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>Over 9.5</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.53585</v>
+        <v>0.4857272727272727</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-115</v>
+        <v>106</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -9680,7 +9680,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 53.6% (fair -115). Your call.</t>
+          <t>Model 48.6% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -9692,17 +9692,17 @@
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>Chicago Cubs @ Milwaukee Brewers</t>
+          <t>Philadelphia Phillies @ New York Mets</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
@@ -9712,17 +9712,17 @@
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.6324196721311476</v>
+        <v>0.5869189189189189</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-172</v>
+        <v>-142</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>-144</v>
+        <v>-122</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -9746,7 +9746,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 63.2% (fair -172). Your call.</t>
+          <t>Model 58.7% (fair -142). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -9923,10 +9923,10 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.4398206278026906</v>
+        <v>0.435695067264574</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H5" s="15" t="n">
         <v>123</v>
@@ -9953,7 +9953,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 44.0% (fair +127). Your call.</t>
+          <t>Model 43.6% (fair +130). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -9989,10 +9989,10 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.560198678414097</v>
+        <v>0.5642828193832599</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-127</v>
+        <v>-130</v>
       </c>
       <c r="H6" s="15" t="n">
         <v>-127</v>
@@ -10019,7 +10019,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 56.0% (fair -127). Your call.</t>
+          <t>Model 56.4% (fair -130). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -10055,10 +10055,10 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5093</v>
+        <v>0.5256</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-104</v>
+        <v>-111</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>125</v>
@@ -10085,7 +10085,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 50.9% (fair -104). Your call.</t>
+          <t>Model 52.6% (fair -111). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -10121,10 +10121,10 @@
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4907</v>
+        <v>0.4744</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="H8" s="15" t="n">
         <v>100</v>
@@ -10151,7 +10151,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 49.1% (fair +104). Your call.</t>
+          <t>Model 47.4% (fair +111). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -10187,10 +10187,10 @@
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.3830384615384615</v>
+        <v>0.3895</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="H9" s="15" t="n">
         <v>160</v>
@@ -10217,7 +10217,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 38.3% (fair +161). Your call.</t>
+          <t>Model 38.9% (fair +157). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -10253,10 +10253,10 @@
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.6169828897338403</v>
+        <v>0.6105372623574145</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-161</v>
+        <v>-157</v>
       </c>
       <c r="H10" s="15" t="n">
         <v>-163</v>
@@ -10283,7 +10283,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 61.7% (fair -161). Your call.</t>
+          <t>Model 61.1% (fair -157). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -10319,10 +10319,10 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.5287686274509803</v>
+        <v>0.5245882352941176</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-112</v>
+        <v>-110</v>
       </c>
       <c r="H11" s="15" t="n">
         <v>-104</v>
@@ -10349,7 +10349,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 52.9% (fair -112). Your call.</t>
+          <t>Model 52.5% (fair -110). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -10385,10 +10385,10 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.4712254901960785</v>
+        <v>0.4753921568627451</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H12" s="15" t="n">
         <v>104</v>
@@ -10415,7 +10415,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 47.1% (fair +112). Your call.</t>
+          <t>Model 47.5% (fair +110). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -10451,10 +10451,10 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5897</v>
+        <v>0.6208</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-144</v>
+        <v>-164</v>
       </c>
       <c r="H13" s="15" t="n">
         <v>117</v>
@@ -10481,7 +10481,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 59.0% (fair -144). Your call.</t>
+          <t>Model 62.1% (fair -164). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -10517,10 +10517,10 @@
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4103</v>
+        <v>0.3792</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>144</v>
+        <v>164</v>
       </c>
       <c r="H14" s="15" t="n">
         <v>111</v>
@@ -10547,7 +10547,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 41.0% (fair +144). Your call.</t>
+          <t>Model 37.9% (fair +164). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -10583,10 +10583,10 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.2759</v>
+        <v>0.2883</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>262</v>
+        <v>247</v>
       </c>
       <c r="H15" s="15" t="n">
         <v>172</v>
@@ -10613,7 +10613,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 27.6% (fair +262). Your call.</t>
+          <t>Model 28.8% (fair +247). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -10649,10 +10649,10 @@
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.7241</v>
+        <v>0.7117</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-262</v>
+        <v>-247</v>
       </c>
       <c r="H16" s="15" t="n">
         <v>156</v>
@@ -10679,7 +10679,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 72.4% (fair -262). Your call.</t>
+          <t>Model 71.2% (fair -247). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -12167,13 +12167,13 @@
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>0.4752863436123348</v>
+        <v>0.4763555555555556</v>
       </c>
       <c r="G39" s="14" t="n">
         <v>110</v>
       </c>
       <c r="H39" s="15" t="n">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="I39" s="13">
         <f>IF($H$39="","",IF($H$39&lt;0,-$H$39/(-$H$39+100),100/($H$39+100)))</f>
@@ -12197,7 +12197,7 @@
       </c>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>Model 47.5% (fair +110). Your call.</t>
+          <t>Model 47.6% (fair +110). Your call.</t>
         </is>
       </c>
       <c r="O39" s="15" t="n"/>
@@ -12233,7 +12233,7 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.5247281938325992</v>
+        <v>0.5236651982378855</v>
       </c>
       <c r="G40" s="14" t="n">
         <v>-110</v>
@@ -12263,7 +12263,7 @@
       </c>
       <c r="N40" s="19" t="inlineStr">
         <is>
-          <t>Model 52.5% (fair -110). Your call.</t>
+          <t>Model 52.4% (fair -110). Your call.</t>
         </is>
       </c>
       <c r="O40" s="15" t="n"/>
@@ -12299,13 +12299,13 @@
         </is>
       </c>
       <c r="F41" s="13" t="n">
-        <v>0.5026</v>
+        <v>0.5031270935960591</v>
       </c>
       <c r="G41" s="14" t="n">
         <v>-101</v>
       </c>
       <c r="H41" s="15" t="n">
-        <v>104</v>
+        <v>-103</v>
       </c>
       <c r="I41" s="13">
         <f>IF($H$41="","",IF($H$41&lt;0,-$H$41/(-$H$41+100),100/($H$41+100)))</f>
@@ -12365,13 +12365,13 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.4974</v>
+        <v>0.4969</v>
       </c>
       <c r="G42" s="14" t="n">
         <v>101</v>
       </c>
       <c r="H42" s="15" t="n">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="I42" s="13">
         <f>IF($H$42="","",IF($H$42&lt;0,-$H$42/(-$H$42+100),100/($H$42+100)))</f>
@@ -12503,7 +12503,7 @@
         <v>-232</v>
       </c>
       <c r="H44" s="15" t="n">
-        <v>-117</v>
+        <v>-118</v>
       </c>
       <c r="I44" s="13">
         <f>IF($H$44="","",IF($H$44&lt;0,-$H$44/(-$H$44+100),100/($H$44+100)))</f>
@@ -12563,13 +12563,13 @@
         </is>
       </c>
       <c r="F45" s="13" t="n">
-        <v>0.4489108910891089</v>
+        <v>0.4483251231527093</v>
       </c>
       <c r="G45" s="14" t="n">
         <v>123</v>
       </c>
       <c r="H45" s="15" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="I45" s="13">
         <f>IF($H$45="","",IF($H$45&lt;0,-$H$45/(-$H$45+100),100/($H$45+100)))</f>
@@ -12593,7 +12593,7 @@
       </c>
       <c r="N45" s="19" t="inlineStr">
         <is>
-          <t>Model 44.9% (fair +123). Your call.</t>
+          <t>Model 44.8% (fair +123). Your call.</t>
         </is>
       </c>
       <c r="O45" s="15" t="n"/>
@@ -12629,7 +12629,7 @@
         </is>
       </c>
       <c r="F46" s="13" t="n">
-        <v>0.5510470588235293</v>
+        <v>0.5517098039215687</v>
       </c>
       <c r="G46" s="14" t="n">
         <v>-123</v>
@@ -12659,7 +12659,7 @@
       </c>
       <c r="N46" s="19" t="inlineStr">
         <is>
-          <t>Model 55.1% (fair -123). Your call.</t>
+          <t>Model 55.2% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O46" s="15" t="n"/>
@@ -12701,7 +12701,7 @@
         <v>-146</v>
       </c>
       <c r="H47" s="15" t="n">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="I47" s="13">
         <f>IF($H$47="","",IF($H$47&lt;0,-$H$47/(-$H$47+100),100/($H$47+100)))</f>
@@ -12959,13 +12959,13 @@
         </is>
       </c>
       <c r="F51" s="13" t="n">
-        <v>0.6197243697478991</v>
+        <v>0.6175531914893617</v>
       </c>
       <c r="G51" s="14" t="n">
-        <v>-163</v>
+        <v>-161</v>
       </c>
       <c r="H51" s="15" t="n">
-        <v>-138</v>
+        <v>-135</v>
       </c>
       <c r="I51" s="13">
         <f>IF($H$51="","",IF($H$51&lt;0,-$H$51/(-$H$51+100),100/($H$51+100)))</f>
@@ -12989,7 +12989,7 @@
       </c>
       <c r="N51" s="19" t="inlineStr">
         <is>
-          <t>Model 62.0% (fair -163). Your call.</t>
+          <t>Model 61.8% (fair -161). Your call.</t>
         </is>
       </c>
       <c r="O51" s="15" t="n"/>
@@ -13025,13 +13025,13 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.3802978723404255</v>
+        <v>0.3824463519313305</v>
       </c>
       <c r="G52" s="14" t="n">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="H52" s="15" t="n">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I52" s="13">
         <f>IF($H$52="","",IF($H$52&lt;0,-$H$52/(-$H$52+100),100/($H$52+100)))</f>
@@ -13055,7 +13055,7 @@
       </c>
       <c r="N52" s="19" t="inlineStr">
         <is>
-          <t>Model 38.0% (fair +163). Your call.</t>
+          <t>Model 38.2% (fair +161). Your call.</t>
         </is>
       </c>
       <c r="O52" s="15" t="n"/>
@@ -13087,17 +13087,17 @@
       </c>
       <c r="E53" s="12" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Over 8</t>
         </is>
       </c>
       <c r="F53" s="13" t="n">
-        <v>0.5473</v>
+        <v>0.4363</v>
       </c>
       <c r="G53" s="14" t="n">
-        <v>-121</v>
+        <v>129</v>
       </c>
       <c r="H53" s="15" t="n">
-        <v>108</v>
+        <v>127</v>
       </c>
       <c r="I53" s="13">
         <f>IF($H$53="","",IF($H$53&lt;0,-$H$53/(-$H$53+100),100/($H$53+100)))</f>
@@ -13121,7 +13121,7 @@
       </c>
       <c r="N53" s="19" t="inlineStr">
         <is>
-          <t>Model 54.7% (fair -121). Your call.</t>
+          <t>Model 43.6% (fair +129). Your call.</t>
         </is>
       </c>
       <c r="O53" s="15" t="n"/>
@@ -13153,17 +13153,17 @@
       </c>
       <c r="E54" s="20" t="inlineStr">
         <is>
-          <t>Under 7.5</t>
+          <t>Under 8</t>
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.4527</v>
+        <v>0.5637</v>
       </c>
       <c r="G54" s="14" t="n">
-        <v>121</v>
+        <v>-129</v>
       </c>
       <c r="H54" s="15" t="n">
-        <v>119</v>
+        <v>-108</v>
       </c>
       <c r="I54" s="13">
         <f>IF($H$54="","",IF($H$54&lt;0,-$H$54/(-$H$54+100),100/($H$54+100)))</f>
@@ -13187,7 +13187,7 @@
       </c>
       <c r="N54" s="19" t="inlineStr">
         <is>
-          <t>Model 45.3% (fair +121). Your call.</t>
+          <t>Model 56.4% (fair -129). Your call.</t>
         </is>
       </c>
       <c r="O54" s="15" t="n"/>
@@ -13351,10 +13351,10 @@
         </is>
       </c>
       <c r="F57" s="13" t="n">
-        <v>0.3676</v>
+        <v>0.36864</v>
       </c>
       <c r="G57" s="14" t="n">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H57" s="15" t="n">
         <v>150</v>
@@ -13381,7 +13381,7 @@
       </c>
       <c r="N57" s="19" t="inlineStr">
         <is>
-          <t>Model 36.8% (fair +172). Your call.</t>
+          <t>Model 36.9% (fair +171). Your call.</t>
         </is>
       </c>
       <c r="O57" s="15" t="n"/>
@@ -13417,13 +13417,13 @@
         </is>
       </c>
       <c r="F58" s="13" t="n">
-        <v>0.6324196721311476</v>
+        <v>0.6313406639004149</v>
       </c>
       <c r="G58" s="14" t="n">
-        <v>-172</v>
+        <v>-171</v>
       </c>
       <c r="H58" s="15" t="n">
-        <v>-144</v>
+        <v>-141</v>
       </c>
       <c r="I58" s="13">
         <f>IF($H$58="","",IF($H$58&lt;0,-$H$58/(-$H$58+100),100/($H$58+100)))</f>
@@ -13447,7 +13447,7 @@
       </c>
       <c r="N58" s="19" t="inlineStr">
         <is>
-          <t>Model 63.2% (fair -172). Your call.</t>
+          <t>Model 63.1% (fair -171). Your call.</t>
         </is>
       </c>
       <c r="O58" s="15" t="n"/>
@@ -13555,7 +13555,7 @@
         <v>167</v>
       </c>
       <c r="H60" s="15" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="I60" s="13">
         <f>IF($H$60="","",IF($H$60&lt;0,-$H$60/(-$H$60+100),100/($H$60+100)))</f>
@@ -13621,7 +13621,7 @@
         <v>106</v>
       </c>
       <c r="H61" s="15" t="n">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="I61" s="13">
         <f>IF($H$61="","",IF($H$61&lt;0,-$H$61/(-$H$61+100),100/($H$61+100)))</f>
@@ -13687,7 +13687,7 @@
         <v>-106</v>
       </c>
       <c r="H62" s="15" t="n">
-        <v>-104</v>
+        <v>-102</v>
       </c>
       <c r="I62" s="13">
         <f>IF($H$62="","",IF($H$62&lt;0,-$H$62/(-$H$62+100),100/($H$62+100)))</f>
@@ -14391,13 +14391,13 @@
         </is>
       </c>
       <c r="F73" s="13" t="n">
-        <v>0.5857560975609757</v>
+        <v>0.6837</v>
       </c>
       <c r="G73" s="14" t="n">
-        <v>-141</v>
+        <v>-216</v>
       </c>
       <c r="H73" s="15" t="n">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="I73" s="13">
         <f>IF($H$73="","",IF($H$73&lt;0,-$H$73/(-$H$73+100),100/($H$73+100)))</f>
@@ -14421,7 +14421,7 @@
       </c>
       <c r="N73" s="19" t="inlineStr">
         <is>
-          <t>Model 58.6% (fair -141). Your call.</t>
+          <t>Model 68.4% (fair -216). Your call.</t>
         </is>
       </c>
       <c r="O73" s="15" t="n"/>
@@ -14457,13 +14457,13 @@
         </is>
       </c>
       <c r="F74" s="13" t="n">
-        <v>0.4142634146341463</v>
+        <v>0.3163</v>
       </c>
       <c r="G74" s="14" t="n">
-        <v>141</v>
+        <v>216</v>
       </c>
       <c r="H74" s="15" t="n">
-        <v>-105</v>
+        <v>105</v>
       </c>
       <c r="I74" s="13">
         <f>IF($H$74="","",IF($H$74&lt;0,-$H$74/(-$H$74+100),100/($H$74+100)))</f>
@@ -14487,7 +14487,7 @@
       </c>
       <c r="N74" s="19" t="inlineStr">
         <is>
-          <t>Model 41.4% (fair +141). Your call.</t>
+          <t>Model 31.6% (fair +216). Your call.</t>
         </is>
       </c>
       <c r="O74" s="15" t="n"/>
@@ -14523,13 +14523,13 @@
         </is>
       </c>
       <c r="F75" s="13" t="n">
-        <v>0.5273809523809523</v>
+        <v>0.5262264150943395</v>
       </c>
       <c r="G75" s="14" t="n">
-        <v>-112</v>
+        <v>-111</v>
       </c>
       <c r="H75" s="15" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I75" s="13">
         <f>IF($H$75="","",IF($H$75&lt;0,-$H$75/(-$H$75+100),100/($H$75+100)))</f>
@@ -14553,7 +14553,7 @@
       </c>
       <c r="N75" s="19" t="inlineStr">
         <is>
-          <t>Model 52.7% (fair -112). Your call.</t>
+          <t>Model 52.6% (fair -111). Your call.</t>
         </is>
       </c>
       <c r="O75" s="15" t="n"/>
@@ -14589,10 +14589,10 @@
         </is>
       </c>
       <c r="F76" s="13" t="n">
-        <v>0.4725818181818182</v>
+        <v>0.4737818181818181</v>
       </c>
       <c r="G76" s="14" t="n">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H76" s="15" t="n">
         <v>-120</v>
@@ -14619,7 +14619,7 @@
       </c>
       <c r="N76" s="19" t="inlineStr">
         <is>
-          <t>Model 47.3% (fair +112). Your call.</t>
+          <t>Model 47.4% (fair +111). Your call.</t>
         </is>
       </c>
       <c r="O76" s="15" t="n"/>
@@ -14859,7 +14859,7 @@
         <v>139</v>
       </c>
       <c r="H80" s="15" t="n">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="I80" s="13">
         <f>IF($H$80="","",IF($H$80&lt;0,-$H$80/(-$H$80+100),100/($H$80+100)))</f>
@@ -14919,13 +14919,13 @@
         </is>
       </c>
       <c r="F81" s="13" t="n">
-        <v>0.4966544117647059</v>
+        <v>0.5008208955223882</v>
       </c>
       <c r="G81" s="14" t="n">
-        <v>101</v>
+        <v>-100</v>
       </c>
       <c r="H81" s="15" t="n">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="I81" s="13">
         <f>IF($H$81="","",IF($H$81&lt;0,-$H$81/(-$H$81+100),100/($H$81+100)))</f>
@@ -14949,7 +14949,7 @@
       </c>
       <c r="N81" s="19" t="inlineStr">
         <is>
-          <t>Model 49.7% (fair +101). Your call.</t>
+          <t>Model 50.1% (fair -100). Your call.</t>
         </is>
       </c>
       <c r="O81" s="15" t="n"/>
@@ -14985,13 +14985,13 @@
         </is>
       </c>
       <c r="F82" s="13" t="n">
-        <v>0.5033571428571428</v>
+        <v>0.4991703703703703</v>
       </c>
       <c r="G82" s="14" t="n">
-        <v>-101</v>
+        <v>100</v>
       </c>
       <c r="H82" s="15" t="n">
-        <v>-180</v>
+        <v>-170</v>
       </c>
       <c r="I82" s="13">
         <f>IF($H$82="","",IF($H$82&lt;0,-$H$82/(-$H$82+100),100/($H$82+100)))</f>
@@ -15015,7 +15015,7 @@
       </c>
       <c r="N82" s="19" t="inlineStr">
         <is>
-          <t>Model 50.3% (fair -101). Your call.</t>
+          <t>Model 49.9% (fair +100). Your call.</t>
         </is>
       </c>
       <c r="O82" s="15" t="n"/>
@@ -15051,10 +15051,10 @@
         </is>
       </c>
       <c r="F83" s="13" t="n">
-        <v>0.4761711711711712</v>
+        <v>0.4748198198198199</v>
       </c>
       <c r="G83" s="14" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H83" s="15" t="n">
         <v>122</v>
@@ -15081,7 +15081,7 @@
       </c>
       <c r="N83" s="19" t="inlineStr">
         <is>
-          <t>Model 47.6% (fair +110). Your call.</t>
+          <t>Model 47.5% (fair +111). Your call.</t>
         </is>
       </c>
       <c r="O83" s="15" t="n"/>
@@ -15117,13 +15117,13 @@
         </is>
       </c>
       <c r="F84" s="13" t="n">
-        <v>0.5238306306306306</v>
+        <v>0.5251666666666667</v>
       </c>
       <c r="G84" s="14" t="n">
-        <v>-110</v>
+        <v>-111</v>
       </c>
       <c r="H84" s="15" t="n">
-        <v>-122</v>
+        <v>-125</v>
       </c>
       <c r="I84" s="13">
         <f>IF($H$84="","",IF($H$84&lt;0,-$H$84/(-$H$84+100),100/($H$84+100)))</f>
@@ -15147,7 +15147,7 @@
       </c>
       <c r="N84" s="19" t="inlineStr">
         <is>
-          <t>Model 52.4% (fair -110). Your call.</t>
+          <t>Model 52.5% (fair -111). Your call.</t>
         </is>
       </c>
       <c r="O84" s="15" t="n"/>
@@ -15315,13 +15315,13 @@
         </is>
       </c>
       <c r="F87" s="13" t="n">
-        <v>0.3390441176470589</v>
+        <v>0.3357142857142857</v>
       </c>
       <c r="G87" s="14" t="n">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="H87" s="15" t="n">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="I87" s="13">
         <f>IF($H$87="","",IF($H$87&lt;0,-$H$87/(-$H$87+100),100/($H$87+100)))</f>
@@ -15345,7 +15345,7 @@
       </c>
       <c r="N87" s="19" t="inlineStr">
         <is>
-          <t>Model 33.9% (fair +195). Your call.</t>
+          <t>Model 33.6% (fair +198). Your call.</t>
         </is>
       </c>
       <c r="O87" s="15" t="n"/>
@@ -15381,10 +15381,10 @@
         </is>
       </c>
       <c r="F88" s="13" t="n">
-        <v>0.6609368421052632</v>
+        <v>0.6643122807017544</v>
       </c>
       <c r="G88" s="14" t="n">
-        <v>-195</v>
+        <v>-198</v>
       </c>
       <c r="H88" s="15" t="n">
         <v>-185</v>
@@ -15411,7 +15411,7 @@
       </c>
       <c r="N88" s="19" t="inlineStr">
         <is>
-          <t>Model 66.1% (fair -195). Your call.</t>
+          <t>Model 66.4% (fair -198). Your call.</t>
         </is>
       </c>
       <c r="O88" s="15" t="n"/>
@@ -15447,7 +15447,7 @@
         </is>
       </c>
       <c r="F89" s="13" t="n">
-        <v>0.5276774774774774</v>
+        <v>0.528281981981982</v>
       </c>
       <c r="G89" s="14" t="n">
         <v>-112</v>
@@ -15513,7 +15513,7 @@
         </is>
       </c>
       <c r="F90" s="13" t="n">
-        <v>0.4723502304147465</v>
+        <v>0.471705069124424</v>
       </c>
       <c r="G90" s="14" t="n">
         <v>112</v>
@@ -15579,7 +15579,7 @@
         </is>
       </c>
       <c r="F91" s="13" t="n">
-        <v>0.5746</v>
+        <v>0.5749</v>
       </c>
       <c r="G91" s="14" t="n">
         <v>-135</v>
@@ -15645,7 +15645,7 @@
         </is>
       </c>
       <c r="F92" s="13" t="n">
-        <v>0.4253658536585366</v>
+        <v>0.4250731707317073</v>
       </c>
       <c r="G92" s="14" t="n">
         <v>135</v>
@@ -15711,10 +15711,10 @@
         </is>
       </c>
       <c r="F93" s="13" t="n">
-        <v>0.6312450980392157</v>
+        <v>0.6276588235294118</v>
       </c>
       <c r="G93" s="14" t="n">
-        <v>-171</v>
+        <v>-169</v>
       </c>
       <c r="H93" s="15" t="n">
         <v>-155</v>
@@ -15741,7 +15741,7 @@
       </c>
       <c r="N93" s="19" t="inlineStr">
         <is>
-          <t>Model 63.1% (fair -171). Your call.</t>
+          <t>Model 62.8% (fair -169). Your call.</t>
         </is>
       </c>
       <c r="O93" s="15" t="n"/>
@@ -15777,13 +15777,13 @@
         </is>
       </c>
       <c r="F94" s="13" t="n">
-        <v>0.3687916666666667</v>
+        <v>0.3723529411764706</v>
       </c>
       <c r="G94" s="14" t="n">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="H94" s="15" t="n">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="I94" s="13">
         <f>IF($H$94="","",IF($H$94&lt;0,-$H$94/(-$H$94+100),100/($H$94+100)))</f>
@@ -15807,7 +15807,7 @@
       </c>
       <c r="N94" s="19" t="inlineStr">
         <is>
-          <t>Model 36.9% (fair +171). Your call.</t>
+          <t>Model 37.2% (fair +169). Your call.</t>
         </is>
       </c>
       <c r="O94" s="15" t="n"/>
@@ -15843,13 +15843,13 @@
         </is>
       </c>
       <c r="F95" s="13" t="n">
-        <v>0.54375</v>
+        <v>0.54865</v>
       </c>
       <c r="G95" s="14" t="n">
-        <v>-119</v>
+        <v>-122</v>
       </c>
       <c r="H95" s="15" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="I95" s="13">
         <f>IF($H$95="","",IF($H$95&lt;0,-$H$95/(-$H$95+100),100/($H$95+100)))</f>
@@ -15873,7 +15873,7 @@
       </c>
       <c r="N95" s="19" t="inlineStr">
         <is>
-          <t>Model 54.4% (fair -119). Your call.</t>
+          <t>Model 54.9% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O95" s="15" t="n"/>
@@ -15909,10 +15909,10 @@
         </is>
       </c>
       <c r="F96" s="13" t="n">
-        <v>0.45625</v>
+        <v>0.45135</v>
       </c>
       <c r="G96" s="14" t="n">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="H96" s="15" t="n">
         <v>100</v>
@@ -15939,7 +15939,7 @@
       </c>
       <c r="N96" s="19" t="inlineStr">
         <is>
-          <t>Model 45.6% (fair +119). Your call.</t>
+          <t>Model 45.1% (fair +122). Your call.</t>
         </is>
       </c>
       <c r="O96" s="15" t="n"/>
@@ -15975,13 +15975,13 @@
         </is>
       </c>
       <c r="F97" s="13" t="n">
-        <v>0.4867788461538461</v>
+        <v>0.4844607843137255</v>
       </c>
       <c r="G97" s="14" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H97" s="15" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="I97" s="13">
         <f>IF($H$97="","",IF($H$97&lt;0,-$H$97/(-$H$97+100),100/($H$97+100)))</f>
@@ -16005,7 +16005,7 @@
       </c>
       <c r="N97" s="19" t="inlineStr">
         <is>
-          <t>Model 48.7% (fair +105). Your call.</t>
+          <t>Model 48.4% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O97" s="15" t="n"/>
@@ -16041,13 +16041,13 @@
         </is>
       </c>
       <c r="F98" s="13" t="n">
-        <v>0.51325</v>
+        <v>0.5154923076923077</v>
       </c>
       <c r="G98" s="14" t="n">
-        <v>-105</v>
+        <v>-106</v>
       </c>
       <c r="H98" s="15" t="n">
-        <v>100</v>
+        <v>-108</v>
       </c>
       <c r="I98" s="13">
         <f>IF($H$98="","",IF($H$98&lt;0,-$H$98/(-$H$98+100),100/($H$98+100)))</f>
@@ -16071,7 +16071,7 @@
       </c>
       <c r="N98" s="19" t="inlineStr">
         <is>
-          <t>Model 51.3% (fair -105). Your call.</t>
+          <t>Model 51.5% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O98" s="15" t="n"/>
@@ -16103,17 +16103,17 @@
       </c>
       <c r="E99" s="12" t="inlineStr">
         <is>
-          <t>Cleveland Guardians +1.5</t>
+          <t>Cleveland Guardians -1.5</t>
         </is>
       </c>
       <c r="F99" s="13" t="n">
-        <v>0.6207610169491526</v>
+        <v>0.2262</v>
       </c>
       <c r="G99" s="14" t="n">
-        <v>-164</v>
+        <v>342</v>
       </c>
       <c r="H99" s="15" t="n">
-        <v>-195</v>
+        <v>165</v>
       </c>
       <c r="I99" s="13">
         <f>IF($H$99="","",IF($H$99&lt;0,-$H$99/(-$H$99+100),100/($H$99+100)))</f>
@@ -16137,7 +16137,7 @@
       </c>
       <c r="N99" s="19" t="inlineStr">
         <is>
-          <t>Model 62.1% (fair -164). Your call.</t>
+          <t>Model 22.6% (fair +342). Your call.</t>
         </is>
       </c>
       <c r="O99" s="15" t="n"/>
@@ -16169,17 +16169,17 @@
       </c>
       <c r="E100" s="20" t="inlineStr">
         <is>
-          <t>Seattle Mariners -1.5</t>
+          <t>Seattle Mariners +1.5</t>
         </is>
       </c>
       <c r="F100" s="13" t="n">
-        <v>0.3792307692307692</v>
+        <v>0.7738</v>
       </c>
       <c r="G100" s="14" t="n">
-        <v>164</v>
+        <v>-342</v>
       </c>
       <c r="H100" s="15" t="n">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="I100" s="13">
         <f>IF($H$100="","",IF($H$100&lt;0,-$H$100/(-$H$100+100),100/($H$100+100)))</f>
@@ -16203,7 +16203,7 @@
       </c>
       <c r="N100" s="19" t="inlineStr">
         <is>
-          <t>Model 37.9% (fair +164). Your call.</t>
+          <t>Model 77.4% (fair -342). Your call.</t>
         </is>
       </c>
       <c r="O100" s="15" t="n"/>
@@ -16503,13 +16503,13 @@
         </is>
       </c>
       <c r="F105" s="13" t="n">
-        <v>0.4248230088495575</v>
+        <v>0.4281363636363636</v>
       </c>
       <c r="G105" s="14" t="n">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H105" s="15" t="n">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="I105" s="13">
         <f>IF($H$105="","",IF($H$105&lt;0,-$H$105/(-$H$105+100),100/($H$105+100)))</f>
@@ -16533,7 +16533,7 @@
       </c>
       <c r="N105" s="19" t="inlineStr">
         <is>
-          <t>Model 42.5% (fair +135). Your call.</t>
+          <t>Model 42.8% (fair +134). Your call.</t>
         </is>
       </c>
       <c r="O105" s="15" t="n"/>
@@ -16569,10 +16569,10 @@
         </is>
       </c>
       <c r="F106" s="13" t="n">
-        <v>0.5751652173913044</v>
+        <v>0.5718304347826088</v>
       </c>
       <c r="G106" s="14" t="n">
-        <v>-135</v>
+        <v>-134</v>
       </c>
       <c r="H106" s="15" t="n">
         <v>-130</v>
@@ -16599,7 +16599,7 @@
       </c>
       <c r="N106" s="19" t="inlineStr">
         <is>
-          <t>Model 57.5% (fair -135). Your call.</t>
+          <t>Model 57.2% (fair -134). Your call.</t>
         </is>
       </c>
       <c r="O106" s="15" t="n"/>
@@ -16635,13 +16635,13 @@
         </is>
       </c>
       <c r="F107" s="13" t="n">
-        <v>0.5891233480176211</v>
+        <v>0.5869189189189189</v>
       </c>
       <c r="G107" s="14" t="n">
-        <v>-143</v>
+        <v>-142</v>
       </c>
       <c r="H107" s="15" t="n">
-        <v>-127</v>
+        <v>-122</v>
       </c>
       <c r="I107" s="13">
         <f>IF($H$107="","",IF($H$107&lt;0,-$H$107/(-$H$107+100),100/($H$107+100)))</f>
@@ -16665,7 +16665,7 @@
       </c>
       <c r="N107" s="19" t="inlineStr">
         <is>
-          <t>Model 58.9% (fair -143). Your call.</t>
+          <t>Model 58.7% (fair -142). Your call.</t>
         </is>
       </c>
       <c r="O107" s="15" t="n"/>
@@ -16701,10 +16701,10 @@
         </is>
       </c>
       <c r="F108" s="13" t="n">
-        <v>0.4108810572687224</v>
+        <v>0.4130837004405286</v>
       </c>
       <c r="G108" s="14" t="n">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="H108" s="15" t="n">
         <v>127</v>
@@ -16731,7 +16731,7 @@
       </c>
       <c r="N108" s="19" t="inlineStr">
         <is>
-          <t>Model 41.1% (fair +143). Your call.</t>
+          <t>Model 41.3% (fair +142). Your call.</t>
         </is>
       </c>
       <c r="O108" s="15" t="n"/>
@@ -16767,10 +16767,10 @@
         </is>
       </c>
       <c r="F109" s="13" t="n">
-        <v>0.4225210084033614</v>
+        <v>0.4236554621848739</v>
       </c>
       <c r="G109" s="14" t="n">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H109" s="15" t="n">
         <v>138</v>
@@ -16797,7 +16797,7 @@
       </c>
       <c r="N109" s="19" t="inlineStr">
         <is>
-          <t>Model 42.3% (fair +137). Your call.</t>
+          <t>Model 42.4% (fair +136). Your call.</t>
         </is>
       </c>
       <c r="O109" s="15" t="n"/>
@@ -16833,13 +16833,13 @@
         </is>
       </c>
       <c r="F110" s="13" t="n">
-        <v>0.5774546218487394</v>
+        <v>0.5763063829787235</v>
       </c>
       <c r="G110" s="14" t="n">
-        <v>-137</v>
+        <v>-136</v>
       </c>
       <c r="H110" s="15" t="n">
-        <v>-138</v>
+        <v>-135</v>
       </c>
       <c r="I110" s="13">
         <f>IF($H$110="","",IF($H$110&lt;0,-$H$110/(-$H$110+100),100/($H$110+100)))</f>
@@ -16863,7 +16863,7 @@
       </c>
       <c r="N110" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -137). Your call.</t>
+          <t>Model 57.6% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O110" s="15" t="n"/>
@@ -16895,7 +16895,7 @@
       </c>
       <c r="E111" s="12" t="inlineStr">
         <is>
-          <t>Over 9.5</t>
+          <t>Over 9</t>
         </is>
       </c>
       <c r="F111" s="13" t="n">
@@ -16961,7 +16961,7 @@
       </c>
       <c r="E112" s="20" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Under 9</t>
         </is>
       </c>
       <c r="F112" s="13" t="n">
@@ -17295,10 +17295,10 @@
         </is>
       </c>
       <c r="F117" s="13" t="n">
-        <v>0.5866682926829269</v>
+        <v>0.6575</v>
       </c>
       <c r="G117" s="14" t="n">
-        <v>-142</v>
+        <v>-192</v>
       </c>
       <c r="H117" s="15" t="n">
         <v>-105</v>
@@ -17325,7 +17325,7 @@
       </c>
       <c r="N117" s="19" t="inlineStr">
         <is>
-          <t>Model 58.7% (fair -142). Your call.</t>
+          <t>Model 65.8% (fair -192). Your call.</t>
         </is>
       </c>
       <c r="O117" s="15" t="n"/>
@@ -17361,13 +17361,13 @@
         </is>
       </c>
       <c r="F118" s="13" t="n">
-        <v>0.4133173076923077</v>
+        <v>0.3425</v>
       </c>
       <c r="G118" s="14" t="n">
-        <v>142</v>
+        <v>192</v>
       </c>
       <c r="H118" s="15" t="n">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="I118" s="13">
         <f>IF($H$118="","",IF($H$118&lt;0,-$H$118/(-$H$118+100),100/($H$118+100)))</f>
@@ -17391,7 +17391,7 @@
       </c>
       <c r="N118" s="19" t="inlineStr">
         <is>
-          <t>Model 41.3% (fair +142). Your call.</t>
+          <t>Model 34.2% (fair +192). Your call.</t>
         </is>
       </c>
       <c r="O118" s="15" t="n"/>
@@ -17427,13 +17427,13 @@
         </is>
       </c>
       <c r="F119" s="13" t="n">
-        <v>0.4223529411764706</v>
+        <v>0.4246800000000001</v>
       </c>
       <c r="G119" s="14" t="n">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="H119" s="15" t="n">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="I119" s="13">
         <f>IF($H$119="","",IF($H$119&lt;0,-$H$119/(-$H$119+100),100/($H$119+100)))</f>
@@ -17457,7 +17457,7 @@
       </c>
       <c r="N119" s="19" t="inlineStr">
         <is>
-          <t>Model 42.2% (fair +137). Your call.</t>
+          <t>Model 42.5% (fair +135). Your call.</t>
         </is>
       </c>
       <c r="O119" s="15" t="n"/>
@@ -17493,10 +17493,10 @@
         </is>
       </c>
       <c r="F120" s="13" t="n">
-        <v>0.5776222222222221</v>
+        <v>0.5752925925925925</v>
       </c>
       <c r="G120" s="14" t="n">
-        <v>-137</v>
+        <v>-135</v>
       </c>
       <c r="H120" s="15" t="n">
         <v>-170</v>
@@ -17523,7 +17523,7 @@
       </c>
       <c r="N120" s="19" t="inlineStr">
         <is>
-          <t>Model 57.8% (fair -137). Your call.</t>
+          <t>Model 57.5% (fair -135). Your call.</t>
         </is>
       </c>
       <c r="O120" s="15" t="n"/>
@@ -18075,13 +18075,13 @@
         </is>
       </c>
       <c r="F129" s="13" t="n">
-        <v>0.5636707317073171</v>
+        <v>0.5606823529411765</v>
       </c>
       <c r="G129" s="14" t="n">
-        <v>-129</v>
+        <v>-128</v>
       </c>
       <c r="H129" s="15" t="n">
-        <v>-105</v>
+        <v>-104</v>
       </c>
       <c r="I129" s="13">
         <f>IF($H$129="","",IF($H$129&lt;0,-$H$129/(-$H$129+100),100/($H$129+100)))</f>
@@ -18105,7 +18105,7 @@
       </c>
       <c r="N129" s="19" t="inlineStr">
         <is>
-          <t>Model 56.4% (fair -129). Your call.</t>
+          <t>Model 56.1% (fair -128). Your call.</t>
         </is>
       </c>
       <c r="O129" s="15" t="n"/>
@@ -18141,13 +18141,13 @@
         </is>
       </c>
       <c r="F130" s="13" t="n">
-        <v>0.4362980769230769</v>
+        <v>0.4393137254901961</v>
       </c>
       <c r="G130" s="14" t="n">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H130" s="15" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="I130" s="13">
         <f>IF($H$130="","",IF($H$130&lt;0,-$H$130/(-$H$130+100),100/($H$130+100)))</f>
@@ -18171,7 +18171,7 @@
       </c>
       <c r="N130" s="19" t="inlineStr">
         <is>
-          <t>Model 43.6% (fair +129). Your call.</t>
+          <t>Model 43.9% (fair +128). Your call.</t>
         </is>
       </c>
       <c r="O130" s="15" t="n"/>
@@ -18207,10 +18207,10 @@
         </is>
       </c>
       <c r="F131" s="13" t="n">
-        <v>0.6019565217391304</v>
+        <v>0.6048391304347827</v>
       </c>
       <c r="G131" s="14" t="n">
-        <v>-151</v>
+        <v>-153</v>
       </c>
       <c r="H131" s="15" t="n">
         <v>-130</v>
@@ -18237,7 +18237,7 @@
       </c>
       <c r="N131" s="19" t="inlineStr">
         <is>
-          <t>Model 60.2% (fair -151). Your call.</t>
+          <t>Model 60.5% (fair -153). Your call.</t>
         </is>
       </c>
       <c r="O131" s="15" t="n"/>
@@ -18273,13 +18273,13 @@
         </is>
       </c>
       <c r="F132" s="13" t="n">
-        <v>0.3980188679245283</v>
+        <v>0.3951612903225807</v>
       </c>
       <c r="G132" s="14" t="n">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="H132" s="15" t="n">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="I132" s="13">
         <f>IF($H$132="","",IF($H$132&lt;0,-$H$132/(-$H$132+100),100/($H$132+100)))</f>
@@ -18303,7 +18303,7 @@
       </c>
       <c r="N132" s="19" t="inlineStr">
         <is>
-          <t>Model 39.8% (fair +151). Your call.</t>
+          <t>Model 39.5% (fair +153). Your call.</t>
         </is>
       </c>
       <c r="O132" s="15" t="n"/>
@@ -18599,13 +18599,13 @@
         </is>
       </c>
       <c r="F137" s="13" t="n">
-        <v>0.6081249999999999</v>
+        <v>0.6065484978540773</v>
       </c>
       <c r="G137" s="14" t="n">
-        <v>-155</v>
+        <v>-154</v>
       </c>
       <c r="H137" s="15" t="n">
-        <v>-140</v>
+        <v>-133</v>
       </c>
       <c r="I137" s="13">
         <f>IF($H$137="","",IF($H$137&lt;0,-$H$137/(-$H$137+100),100/($H$137+100)))</f>
@@ -18629,7 +18629,7 @@
       </c>
       <c r="N137" s="19" t="inlineStr">
         <is>
-          <t>Model 60.8% (fair -155). Your call.</t>
+          <t>Model 60.7% (fair -154). Your call.</t>
         </is>
       </c>
       <c r="O137" s="15" t="n"/>
@@ -18665,13 +18665,13 @@
         </is>
       </c>
       <c r="F138" s="13" t="n">
-        <v>0.3918636363636363</v>
+        <v>0.3934234234234235</v>
       </c>
       <c r="G138" s="14" t="n">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="H138" s="15" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I138" s="13">
         <f>IF($H$138="","",IF($H$138&lt;0,-$H$138/(-$H$138+100),100/($H$138+100)))</f>
@@ -18695,7 +18695,7 @@
       </c>
       <c r="N138" s="19" t="inlineStr">
         <is>
-          <t>Model 39.2% (fair +155). Your call.</t>
+          <t>Model 39.3% (fair +154). Your call.</t>
         </is>
       </c>
       <c r="O138" s="15" t="n"/>
@@ -18731,10 +18731,10 @@
         </is>
       </c>
       <c r="F139" s="13" t="n">
-        <v>0.5442</v>
+        <v>0.5396</v>
       </c>
       <c r="G139" s="14" t="n">
-        <v>-119</v>
+        <v>-117</v>
       </c>
       <c r="H139" s="15" t="n"/>
       <c r="I139" s="13">
@@ -18759,7 +18759,7 @@
       </c>
       <c r="N139" s="19" t="inlineStr">
         <is>
-          <t>Model 54.4% (fair -119). Your call.</t>
+          <t>Model 54.0% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O139" s="15" t="n"/>
@@ -18795,10 +18795,10 @@
         </is>
       </c>
       <c r="F140" s="13" t="n">
-        <v>0.4558013215859031</v>
+        <v>0.460388986784141</v>
       </c>
       <c r="G140" s="14" t="n">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H140" s="15" t="n">
         <v>-127</v>
@@ -18825,7 +18825,7 @@
       </c>
       <c r="N140" s="19" t="inlineStr">
         <is>
-          <t>Model 45.6% (fair +119). Your call.</t>
+          <t>Model 46.0% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O140" s="15" t="n"/>
@@ -18861,10 +18861,10 @@
         </is>
       </c>
       <c r="F141" s="13" t="n">
-        <v>0.4827439024390244</v>
+        <v>0.4466</v>
       </c>
       <c r="G141" s="14" t="n">
-        <v>107</v>
+        <v>124</v>
       </c>
       <c r="H141" s="15" t="n">
         <v>-105</v>
@@ -18891,7 +18891,7 @@
       </c>
       <c r="N141" s="19" t="inlineStr">
         <is>
-          <t>Model 48.3% (fair +107). Your call.</t>
+          <t>Model 44.7% (fair +124). Your call.</t>
         </is>
       </c>
       <c r="O141" s="15" t="n"/>
@@ -18927,13 +18927,13 @@
         </is>
       </c>
       <c r="F142" s="13" t="n">
-        <v>0.5172596153846154</v>
+        <v>0.5534</v>
       </c>
       <c r="G142" s="14" t="n">
-        <v>-107</v>
+        <v>-124</v>
       </c>
       <c r="H142" s="15" t="n">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="I142" s="13">
         <f>IF($H$142="","",IF($H$142&lt;0,-$H$142/(-$H$142+100),100/($H$142+100)))</f>
@@ -18957,7 +18957,7 @@
       </c>
       <c r="N142" s="19" t="inlineStr">
         <is>
-          <t>Model 51.7% (fair -107). Your call.</t>
+          <t>Model 55.3% (fair -124). Your call.</t>
         </is>
       </c>
       <c r="O142" s="15" t="n"/>
@@ -18993,13 +18993,13 @@
         </is>
       </c>
       <c r="F143" s="13" t="n">
-        <v>0.2867058823529413</v>
+        <v>0.2826</v>
       </c>
       <c r="G143" s="14" t="n">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="H143" s="15" t="n">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="I143" s="13">
         <f>IF($H$143="","",IF($H$143&lt;0,-$H$143/(-$H$143+100),100/($H$143+100)))</f>
@@ -19023,7 +19023,7 @@
       </c>
       <c r="N143" s="19" t="inlineStr">
         <is>
-          <t>Model 28.7% (fair +249). Your call.</t>
+          <t>Model 28.3% (fair +254). Your call.</t>
         </is>
       </c>
       <c r="O143" s="15" t="n"/>
@@ -19059,10 +19059,10 @@
         </is>
       </c>
       <c r="F144" s="13" t="n">
-        <v>0.7133</v>
+        <v>0.7174</v>
       </c>
       <c r="G144" s="14" t="n">
-        <v>-249</v>
+        <v>-254</v>
       </c>
       <c r="H144" s="15" t="n"/>
       <c r="I144" s="13">
@@ -19087,7 +19087,7 @@
       </c>
       <c r="N144" s="19" t="inlineStr">
         <is>
-          <t>Model 71.3% (fair -249). Your call.</t>
+          <t>Model 71.7% (fair -254). Your call.</t>
         </is>
       </c>
       <c r="O144" s="15" t="n"/>
@@ -19264,7 +19264,7 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.2905507246376811</v>
+        <v>0.2906666666666666</v>
       </c>
       <c r="G5" s="14" t="n">
         <v>244</v>
@@ -19330,13 +19330,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.7094504273504273</v>
+        <v>0.7092857142857143</v>
       </c>
       <c r="G6" s="14" t="n">
         <v>-244</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-251</v>
+        <v>-250</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -19392,14 +19392,14 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 179.5</t>
+          <t>Over 181.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.715</v>
+        <v>0.6680980392156862</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-251</v>
+        <v>-201</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>-104</v>
@@ -19426,7 +19426,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 71.5% (fair -251). Your call.</t>
+          <t>Model 66.8% (fair -201). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -19458,14 +19458,14 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 179.5</t>
+          <t>Under 181.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.285</v>
+        <v>0.3319</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>251</v>
+        <v>201</v>
       </c>
       <c r="H8" s="15" t="n">
         <v>-104</v>
@@ -19492,7 +19492,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 28.5% (fair +251). Your call.</t>
+          <t>Model 33.2% (fair +201). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -19524,14 +19524,14 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Indiana Fever -6.5</t>
+          <t>Indiana Fever -7.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.513</v>
+        <v>0.4974749999999999</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-105</v>
+        <v>101</v>
       </c>
       <c r="H9" s="15" t="n">
         <v>-108</v>
@@ -19558,7 +19558,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 51.3% (fair -105). Your call.</t>
+          <t>Model 49.7% (fair +101). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -19590,17 +19590,17 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks +6.5</t>
+          <t>Los Angeles Sparks +7.5</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.4869756097560976</v>
+        <v>0.5024999999999999</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>105</v>
+        <v>-101</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -19624,7 +19624,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 48.7% (fair +105). Your call.</t>
+          <t>Model 50.2% (fair -101). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -19660,13 +19660,13 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.7612197530864198</v>
+        <v>0.7708850574712643</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-319</v>
+        <v>-336</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>-305</v>
+        <v>-335</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -19690,7 +19690,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 76.1% (fair -319). Your call.</t>
+          <t>Model 77.1% (fair -336). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -19726,13 +19726,13 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.238825</v>
+        <v>0.2291494252873564</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>319</v>
+        <v>336</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>300</v>
+        <v>335</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -19756,7 +19756,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 23.9% (fair +319). Your call.</t>
+          <t>Model 22.9% (fair +336). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -19930,7 +19930,7 @@
         <v>439</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>410</v>
+        <v>430</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -19996,7 +19996,7 @@
         <v>-439</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -20056,10 +20056,10 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.6274734375000001</v>
+        <v>0.6261328125000001</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-168</v>
+        <v>-167</v>
       </c>
       <c r="H17" s="15" t="n">
         <v>-156</v>
@@ -20086,7 +20086,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 62.7% (fair -168). Your call.</t>
+          <t>Model 62.6% (fair -167). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -20122,13 +20122,13 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.3725095057034221</v>
+        <v>0.3738846153846154</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -20152,7 +20152,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 37.3% (fair +168). Your call.</t>
+          <t>Model 37.4% (fair +167). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -20320,13 +20320,13 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.5042</v>
+        <v>0.5099926829268293</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>-102</v>
+        <v>-104</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>113</v>
+        <v>-105</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -20350,7 +20350,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 50.4% (fair -102). Your call.</t>
+          <t>Model 51.0% (fair -104). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -20386,10 +20386,10 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.4958</v>
+        <v>0.49</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H22" s="15" t="n">
         <v>108</v>
@@ -20416,7 +20416,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 49.6% (fair +102). Your call.</t>
+          <t>Model 49.0% (fair +104). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -20452,10 +20452,10 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.3029129129129129</v>
+        <v>0.3044444444444445</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="H23" s="15" t="n">
         <v>233</v>
@@ -20482,7 +20482,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 30.3% (fair +230). Your call.</t>
+          <t>Model 30.4% (fair +228). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -20518,13 +20518,13 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.6970782608695653</v>
+        <v>0.6955714714714715</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-230</v>
+        <v>-228</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>-245</v>
+        <v>-233</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -20548,7 +20548,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 69.7% (fair -230). Your call.</t>
+          <t>Model 69.6% (fair -228). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -20848,10 +20848,10 @@
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.7520298701298702</v>
+        <v>0.7484025974025973</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-303</v>
+        <v>-297</v>
       </c>
       <c r="H29" s="15" t="n">
         <v>-285</v>
@@ -20878,7 +20878,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 75.2% (fair -303). Your call.</t>
+          <t>Model 74.8% (fair -297). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -20914,13 +20914,13 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.247975</v>
+        <v>0.2516103896103896</v>
       </c>
       <c r="G30" s="14" t="n">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>300</v>
+        <v>285</v>
       </c>
       <c r="I30" s="13">
         <f>IF($H$30="","",IF($H$30&lt;0,-$H$30/(-$H$30+100),100/($H$30+100)))</f>
@@ -20944,7 +20944,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Model 24.8% (fair +303). Your call.</t>
+          <t>Model 25.2% (fair +297). Your call.</t>
         </is>
       </c>
       <c r="O30" s="15" t="n"/>
@@ -21112,13 +21112,13 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.5767615384615384</v>
+        <v>0.5778666666666666</v>
       </c>
       <c r="G33" s="14" t="n">
-        <v>-136</v>
+        <v>-137</v>
       </c>
       <c r="H33" s="15" t="n">
-        <v>-108</v>
+        <v>-110</v>
       </c>
       <c r="I33" s="13">
         <f>IF($H$33="","",IF($H$33&lt;0,-$H$33/(-$H$33+100),100/($H$33+100)))</f>
@@ -21142,7 +21142,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>Model 57.7% (fair -136). Your call.</t>
+          <t>Model 57.8% (fair -137). Your call.</t>
         </is>
       </c>
       <c r="O33" s="15" t="n"/>
@@ -21178,10 +21178,10 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.4232380952380952</v>
+        <v>0.4221380952380953</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H34" s="15" t="n">
         <v>-110</v>
@@ -21208,7 +21208,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>Model 42.3% (fair +136). Your call.</t>
+          <t>Model 42.2% (fair +137). Your call.</t>
         </is>
       </c>
       <c r="O34" s="15" t="n"/>
@@ -21504,17 +21504,17 @@
       </c>
       <c r="E39" s="12" t="inlineStr">
         <is>
-          <t>Golden State Valkyries +1.5</t>
+          <t>Golden State Valkyries -1.5</t>
         </is>
       </c>
       <c r="F39" s="13" t="n">
-        <v>0.5795450980392156</v>
+        <v>0.5218536585365855</v>
       </c>
       <c r="G39" s="14" t="n">
-        <v>-138</v>
+        <v>-109</v>
       </c>
       <c r="H39" s="15" t="n">
-        <v>-104</v>
+        <v>105</v>
       </c>
       <c r="I39" s="13">
         <f>IF($H$39="","",IF($H$39&lt;0,-$H$39/(-$H$39+100),100/($H$39+100)))</f>
@@ -21538,7 +21538,7 @@
       </c>
       <c r="N39" s="19" t="inlineStr">
         <is>
-          <t>Model 58.0% (fair -138). Your call.</t>
+          <t>Model 52.2% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O39" s="15" t="n"/>
@@ -21570,17 +21570,17 @@
       </c>
       <c r="E40" s="20" t="inlineStr">
         <is>
-          <t>New York Liberty -1.5</t>
+          <t>New York Liberty +1.5</t>
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.4204878048780488</v>
+        <v>0.4781188118811881</v>
       </c>
       <c r="G40" s="14" t="n">
-        <v>138</v>
+        <v>109</v>
       </c>
       <c r="H40" s="15" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="I40" s="13">
         <f>IF($H$40="","",IF($H$40&lt;0,-$H$40/(-$H$40+100),100/($H$40+100)))</f>
@@ -21604,7 +21604,7 @@
       </c>
       <c r="N40" s="19" t="inlineStr">
         <is>
-          <t>Model 42.0% (fair +138). Your call.</t>
+          <t>Model 47.8% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O40" s="15" t="n"/>

</xml_diff>